<commit_message>
Refresh supervisor for Etsy live batch
</commit_message>
<xml_diff>
--- a/Database/Unified_Listing_Registry.xlsx
+++ b/Database/Unified_Listing_Registry.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Unified Registry" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Unified Registry'!$A$1:$T$274</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Unified Registry'!$A$1:$T$275</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T274"/>
+  <dimension ref="A1:T275"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -748,8 +748,16 @@
           <t>69f192aa5ea38382140f1d7b</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>406892408950</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406892408950</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>4pc Kiss-Cut Sticker Set Mechanical Raven Familiar Laptop Journal Bottle Dark</t>
@@ -760,9 +768,21 @@
           <t>$11.99</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M5" t="b">
         <v>0</v>
       </c>
@@ -786,7 +806,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -2168,8 +2188,16 @@
           <t>69f1b00840c796ee97058144</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>406892414116</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406892414116</t>
+        </is>
+      </c>
       <c r="H26" t="inlineStr">
         <is>
           <t>Floating Island Sanctuary 4pc 6x6 Kiss-Cut Sticker Zen Aesthetic Laptop Journal</t>
@@ -2180,9 +2208,21 @@
           <t>$11.99</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M26" t="b">
         <v>0</v>
       </c>
@@ -2206,7 +2246,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -2560,7 +2600,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PublishExternalPending_Mockups4</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -2760,7 +2800,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PublishExternalPending_Mockups4</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2892,7 +2932,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PublishExternalPending_Mockups4</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2960,7 +3000,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PublishExternalPending_Mockups4</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3092,7 +3132,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PublishExternalPending_Mockups4</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3160,7 +3200,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PublishExternalPending_Mockups4</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -3228,7 +3268,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PublishExternalPending_Mockups4</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -3296,7 +3336,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PublishExternalPending_Mockups4</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -3364,7 +3404,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PublishExternalPending_Mockups4</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -3496,7 +3536,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PublishExternalPending_Mockups4</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -3708,8 +3748,16 @@
           <t>69f2396ccaeb1241880b692d</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>406902622710</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902622710</t>
+        </is>
+      </c>
       <c r="H49" t="inlineStr">
         <is>
           <t>Zen Aesthetic Dragon Coil 4pc 6x6 Kiss-Cut Sticker Laptop Journal Water Bottle</t>
@@ -3720,9 +3768,21 @@
           <t>$11.99</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M49" t="b">
         <v>0</v>
       </c>
@@ -3746,7 +3806,7 @@
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -3776,8 +3836,16 @@
           <t>69f21a5da7777da1970fd378</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>406902640998</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902640998</t>
+        </is>
+      </c>
       <c r="H50" t="inlineStr">
         <is>
           <t>Floating Dragon Minimal Zen 4pc 6x6 Kiss-Cut Vinyl Desk Collector Decor Sky Art</t>
@@ -3788,9 +3856,21 @@
           <t>$11.99</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M50" t="b">
         <v>0</v>
       </c>
@@ -3814,7 +3894,7 @@
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -3844,8 +3924,16 @@
           <t>69f21b07b0d6b88b2805ebe3</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>406902663232</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902663232</t>
+        </is>
+      </c>
       <c r="H51" t="inlineStr">
         <is>
           <t>Zen Aesthetic Dragon and Pearl 4pc 6x6 Kiss-Cut Sticker Laptop Journal Water</t>
@@ -3856,9 +3944,21 @@
           <t>$11.99</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M51" t="b">
         <v>0</v>
       </c>
@@ -3882,7 +3982,7 @@
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -3904,7 +4004,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PublishExternalPending_Mockups4</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -3980,8 +4080,16 @@
           <t>69f23a2fa7777da1970fe60d</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>406902713267</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902713267</t>
+        </is>
+      </c>
       <c r="H53" t="inlineStr">
         <is>
           <t>Sleeping Dragon Minimal Zen 4pc 6x6 Kiss-Cut Vinyl Desk Collector Decor Laptop</t>
@@ -3992,9 +4100,21 @@
           <t>$11.99</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M53" t="b">
         <v>0</v>
       </c>
@@ -4018,7 +4138,7 @@
       </c>
       <c r="T53" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -4048,8 +4168,16 @@
           <t>69f23a99c326d7da170bfe8d</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>406902886081</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902886081</t>
+        </is>
+      </c>
       <c r="H54" t="inlineStr">
         <is>
           <t>Translucent Jade Dragon Mindful Zen 4pc 6x6 Vinyl Sticker Yoga Minimalist Gift</t>
@@ -4060,9 +4188,21 @@
           <t>$11.99</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M54" t="b">
         <v>0</v>
       </c>
@@ -4086,7 +4226,7 @@
       </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -4116,8 +4256,16 @@
           <t>69f23b5ce64c9f31b70f415b</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>406902889638</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902889638</t>
+        </is>
+      </c>
       <c r="H55" t="inlineStr">
         <is>
           <t>Kintsugi Gold Dragon Mindful Zen 4pc 6x6 Vinyl Sticker Yoga Minimalist Gift</t>
@@ -4128,9 +4276,21 @@
           <t>$11.99</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M55" t="b">
         <v>0</v>
       </c>
@@ -4154,7 +4314,7 @@
       </c>
       <c r="T55" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -4184,8 +4344,16 @@
           <t>69f23c10caeb1241880b6afe</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>406902896387</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902896387</t>
+        </is>
+      </c>
       <c r="H56" t="inlineStr">
         <is>
           <t>Bioluminescent Dragon 4pc 6x6 Kiss-Cut Sticker Zen Aesthetic Laptop Journal</t>
@@ -4196,9 +4364,21 @@
           <t>$11.99</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M56" t="b">
         <v>0</v>
       </c>
@@ -4222,7 +4402,7 @@
       </c>
       <c r="T56" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -4252,8 +4432,16 @@
           <t>69f252f4357398ded80f61c9</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>406902900109</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902900109</t>
+        </is>
+      </c>
       <c r="H57" t="inlineStr">
         <is>
           <t>Crystalline Dragon Minimal Zen 4pc 6x6 Kiss-Cut Vinyl Desk Collector Decor Gift</t>
@@ -4264,9 +4452,21 @@
           <t>$11.99</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M57" t="b">
         <v>0</v>
       </c>
@@ -4290,7 +4490,7 @@
       </c>
       <c r="T57" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -4320,8 +4520,16 @@
           <t>69f253bc357398ded80f6242</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>406903032635</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903032635</t>
+        </is>
+      </c>
       <c r="H58" t="inlineStr">
         <is>
           <t>Dragon Meditation Minimal Zen 4pc 6x6 Kiss-Cut Vinyl Desk Collector Decor Gift</t>
@@ -4332,9 +4540,21 @@
           <t>$11.99</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr"/>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M58" t="b">
         <v>0</v>
       </c>
@@ -4358,7 +4578,7 @@
       </c>
       <c r="T58" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -4388,8 +4608,16 @@
           <t>69f2547229c1d0349a00e796</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr"/>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>406903037933</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903037933</t>
+        </is>
+      </c>
       <c r="H59" t="inlineStr">
         <is>
           <t>Mindful Zen Azure Dragon Warrior 4pc 6x6 Vinyl Sticker Laptop Journal Gift Desk</t>
@@ -4400,9 +4628,21 @@
           <t>$11.99</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr"/>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M59" t="b">
         <v>0</v>
       </c>
@@ -4426,7 +4666,7 @@
       </c>
       <c r="T59" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -4456,8 +4696,16 @@
           <t>69f25526ad218fe47f0cc0d3</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>406903041315</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903041315</t>
+        </is>
+      </c>
       <c r="H60" t="inlineStr">
         <is>
           <t>Dragon Cherry Blossom 4pc 6x6 Kiss-Cut Sticker Zen Aesthetic Laptop Journal</t>
@@ -4468,9 +4716,21 @@
           <t>$11.99</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M60" t="b">
         <v>0</v>
       </c>
@@ -4494,7 +4754,7 @@
       </c>
       <c r="T60" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -4524,8 +4784,16 @@
           <t>69f255dae64c9f31b70f4ea6</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr"/>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>406903044643</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903044643</t>
+        </is>
+      </c>
       <c r="H61" t="inlineStr">
         <is>
           <t>Moonlit Dragon 4pc 6x6 Kiss-Cut Sticker Zen Aesthetic Laptop Journal Desk Decor</t>
@@ -4536,9 +4804,21 @@
           <t>$11.99</t>
         </is>
       </c>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr"/>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M61" t="b">
         <v>0</v>
       </c>
@@ -4562,7 +4842,7 @@
       </c>
       <c r="T61" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -4592,8 +4872,16 @@
           <t>69f259bc5f78c14a7b0a4760</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>406903049411</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903049411</t>
+        </is>
+      </c>
       <c r="H62" t="inlineStr">
         <is>
           <t>Minimal Zen Dragon Calligraphy 4pc 6x6 Sticker Sheet Serene Mindful Clean Decor</t>
@@ -4604,9 +4892,21 @@
           <t>$11.99</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr"/>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M62" t="b">
         <v>0</v>
       </c>
@@ -4630,7 +4930,7 @@
       </c>
       <c r="T62" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -4660,8 +4960,16 @@
           <t>69f25a86a7777da1970ff5f3</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>406903249053</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903249053</t>
+        </is>
+      </c>
       <c r="H63" t="inlineStr">
         <is>
           <t>Minimal Zen Translucent Jade Dragon 4pc 6x6 Sticker Sheet Serene Mindful Clean</t>
@@ -4672,9 +4980,21 @@
           <t>$11.99</t>
         </is>
       </c>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M63" t="b">
         <v>0</v>
       </c>
@@ -4698,7 +5018,7 @@
       </c>
       <c r="T63" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -4728,8 +5048,16 @@
           <t>69f25b3ce64c9f31b70f50ed</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>406903249987</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903249987</t>
+        </is>
+      </c>
       <c r="H64" t="inlineStr">
         <is>
           <t>Minimal Zen Kintsugi Gold Dragon 4pc 6x6 Sticker Sheet Serene Mindful Calm Gift</t>
@@ -4796,8 +5124,16 @@
           <t>69f25bee9b469f716d0e7056</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr"/>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>406903250891</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903250891</t>
+        </is>
+      </c>
       <c r="H65" t="inlineStr">
         <is>
           <t>Zen Aesthetic Bioluminescent Dragon 4pc 6x6 Kiss-Cut Sticker Laptop Journal</t>
@@ -4864,8 +5200,16 @@
           <t>69f25ca39577aaffd5066a80</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr"/>
-      <c r="G66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>406903252007</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903252007</t>
+        </is>
+      </c>
       <c r="H66" t="inlineStr">
         <is>
           <t>Crystalline Dragon Core 4pc 6x6 Kiss-Cut Sticker Zen Aesthetic Laptop Journal</t>
@@ -4932,8 +5276,16 @@
           <t>69f25d56c326d7da170c0f79</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>406903252739</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903252739</t>
+        </is>
+      </c>
       <c r="H67" t="inlineStr">
         <is>
           <t>Golden Vein Circuitry Dragon 4pc 6x6 Kiss-Cut Sticker Zen Aesthetic Laptop Gift</t>
@@ -4992,7 +5344,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PublishExternalPending_Mockups4</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -5060,7 +5412,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PublishExternalPending_Mockups4</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -5136,8 +5488,16 @@
           <t>69f26062cd8d04605103d10b</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr"/>
-      <c r="G70" t="inlineStr"/>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>406903753067</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903753067</t>
+        </is>
+      </c>
       <c r="H70" t="inlineStr">
         <is>
           <t>Minimal Zen Dragon Guardian 4pc 6x6 Sticker Sheet Serene Mindful Clean Decor</t>
@@ -5204,8 +5564,16 @@
           <t>69f261185f78c14a7b0a4b29</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr"/>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>406903757240</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903757240</t>
+        </is>
+      </c>
       <c r="H71" t="inlineStr">
         <is>
           <t>Minimal Zen Jade Phoenix Ascension 4pc 6x6 Sticker Sheet Serene Mindful Clean</t>
@@ -5272,8 +5640,16 @@
           <t>69f261cd5269e3325904b816</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr"/>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>406903762328</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903762328</t>
+        </is>
+      </c>
       <c r="H72" t="inlineStr">
         <is>
           <t>Zen Aesthetic Lotus Lantern Vessel 4pc 6x6 Kiss-Cut Sticker Laptop Journal Gift</t>
@@ -10396,8 +10772,16 @@
           <t>69f28800cd8d04605103e53a</t>
         </is>
       </c>
-      <c r="F151" t="inlineStr"/>
-      <c r="G151" t="inlineStr"/>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>406902584620</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902584620</t>
+        </is>
+      </c>
       <c r="H151" t="inlineStr">
         <is>
           <t>Celestial Gateway Dark Academia Poster 12x18 Study Decor Moonstone Architecture</t>
@@ -10408,9 +10792,21 @@
           <t>$34.99</t>
         </is>
       </c>
-      <c r="J151" t="inlineStr"/>
-      <c r="K151" t="inlineStr"/>
-      <c r="L151" t="inlineStr"/>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M151" t="b">
         <v>0</v>
       </c>
@@ -10434,7 +10830,7 @@
       </c>
       <c r="T151" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Has_View_Monitor</t>
         </is>
       </c>
     </row>
@@ -10464,8 +10860,16 @@
           <t>69f2906f7f1017d51b0d5f76</t>
         </is>
       </c>
-      <c r="F152" t="inlineStr"/>
-      <c r="G152" t="inlineStr"/>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>406902600741</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902600741</t>
+        </is>
+      </c>
       <c r="H152" t="inlineStr">
         <is>
           <t>Dark Academia Obsidian Threshold Poster 12x18 Vintage Study Decor Mentor Wisdom</t>
@@ -10476,9 +10880,21 @@
           <t>$34.99</t>
         </is>
       </c>
-      <c r="J152" t="inlineStr"/>
-      <c r="K152" t="inlineStr"/>
-      <c r="L152" t="inlineStr"/>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M152" t="b">
         <v>0</v>
       </c>
@@ -10502,7 +10918,7 @@
       </c>
       <c r="T152" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -10532,8 +10948,16 @@
           <t>69f29152357398ded80f8178</t>
         </is>
       </c>
-      <c r="F153" t="inlineStr"/>
-      <c r="G153" t="inlineStr"/>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>406902616799</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902616799</t>
+        </is>
+      </c>
       <c r="H153" t="inlineStr">
         <is>
           <t>Dark Academia Serpentine Portal of Alchemical Texts 12x18 Poster Study Decor</t>
@@ -10544,9 +10968,21 @@
           <t>$34.99</t>
         </is>
       </c>
-      <c r="J153" t="inlineStr"/>
-      <c r="K153" t="inlineStr"/>
-      <c r="L153" t="inlineStr"/>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M153" t="b">
         <v>1</v>
       </c>
@@ -10578,7 +11014,7 @@
       </c>
       <c r="T153" t="inlineStr">
         <is>
-          <t>Etsy_Draft_Prepared</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -10608,8 +11044,16 @@
           <t>69f298dc9577aaffd50689b0</t>
         </is>
       </c>
-      <c r="F154" t="inlineStr"/>
-      <c r="G154" t="inlineStr"/>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>406902588642</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902588642</t>
+        </is>
+      </c>
       <c r="H154" t="inlineStr">
         <is>
           <t>Astrolabe Compass Ritual Disc Dark Academia 5x7 Acrylic Art Study Decor Shelf</t>
@@ -10620,9 +11064,21 @@
           <t>$89.99</t>
         </is>
       </c>
-      <c r="J154" t="inlineStr"/>
-      <c r="K154" t="inlineStr"/>
-      <c r="L154" t="inlineStr"/>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M154" t="b">
         <v>1</v>
       </c>
@@ -10654,7 +11110,7 @@
       </c>
       <c r="T154" t="inlineStr">
         <is>
-          <t>Etsy_Draft_Prepared</t>
+          <t>Published_Has_View_Monitor</t>
         </is>
       </c>
     </row>
@@ -10684,8 +11140,16 @@
           <t>69f299c1a3119247600cbe18</t>
         </is>
       </c>
-      <c r="F155" t="inlineStr"/>
-      <c r="G155" t="inlineStr"/>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>406902606976</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902606976</t>
+        </is>
+      </c>
       <c r="H155" t="inlineStr">
         <is>
           <t>Plague Doctor Raven Skull Grimdark Alchemy 5x7 Acrylic Art Block Collectible</t>
@@ -10696,9 +11160,21 @@
           <t>$89.99</t>
         </is>
       </c>
-      <c r="J155" t="inlineStr"/>
-      <c r="K155" t="inlineStr"/>
-      <c r="L155" t="inlineStr"/>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M155" t="b">
         <v>0</v>
       </c>
@@ -10722,7 +11198,7 @@
       </c>
       <c r="T155" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -10752,8 +11228,16 @@
           <t>69f29a72c411a56f6902930d</t>
         </is>
       </c>
-      <c r="F156" t="inlineStr"/>
-      <c r="G156" t="inlineStr"/>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>406902620519</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902620519</t>
+        </is>
+      </c>
       <c r="H156" t="inlineStr">
         <is>
           <t>Zen Mechanical Crane 5x7 Acrylic Block Desk Art Calm Decor Origami Sculpture</t>
@@ -10764,9 +11248,21 @@
           <t>$89.99</t>
         </is>
       </c>
-      <c r="J156" t="inlineStr"/>
-      <c r="K156" t="inlineStr"/>
-      <c r="L156" t="inlineStr"/>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M156" t="b">
         <v>1</v>
       </c>
@@ -10798,7 +11294,7 @@
       </c>
       <c r="T156" t="inlineStr">
         <is>
-          <t>Etsy_Draft_Prepared</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -10828,8 +11324,16 @@
           <t>69f29fe09577aaffd5068e03</t>
         </is>
       </c>
-      <c r="F157" t="inlineStr"/>
-      <c r="G157" t="inlineStr"/>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>406902627420</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902627420</t>
+        </is>
+      </c>
       <c r="H157" t="inlineStr">
         <is>
           <t>Celestial Armillary Sphere Dark Academia Poster 12x18 Scholar Study Decor Wall</t>
@@ -10840,9 +11344,21 @@
           <t>$34.99</t>
         </is>
       </c>
-      <c r="J157" t="inlineStr"/>
-      <c r="K157" t="inlineStr"/>
-      <c r="L157" t="inlineStr"/>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M157" t="b">
         <v>1</v>
       </c>
@@ -10874,7 +11390,7 @@
       </c>
       <c r="T157" t="inlineStr">
         <is>
-          <t>Etsy_Draft_Prepared</t>
+          <t>Published_Has_View_Monitor</t>
         </is>
       </c>
     </row>
@@ -10904,8 +11420,16 @@
           <t>69f2a0cacaeb1241880b9e8d</t>
         </is>
       </c>
-      <c r="F158" t="inlineStr"/>
-      <c r="G158" t="inlineStr"/>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>406902648209</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902648209</t>
+        </is>
+      </c>
       <c r="H158" t="inlineStr">
         <is>
           <t>Celestial Armillary Codex Academia Poster 12x18 Vintage Astronomy Decor Wall</t>
@@ -10916,9 +11440,21 @@
           <t>$34.99</t>
         </is>
       </c>
-      <c r="J158" t="inlineStr"/>
-      <c r="K158" t="inlineStr"/>
-      <c r="L158" t="inlineStr"/>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M158" t="b">
         <v>0</v>
       </c>
@@ -10942,7 +11478,7 @@
       </c>
       <c r="T158" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Has_View_Monitor</t>
         </is>
       </c>
     </row>
@@ -10972,8 +11508,16 @@
           <t>69f2a1b8a7777da197101a96</t>
         </is>
       </c>
-      <c r="F159" t="inlineStr"/>
-      <c r="G159" t="inlineStr"/>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>406902669660</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902669660</t>
+        </is>
+      </c>
       <c r="H159" t="inlineStr">
         <is>
           <t>Academia Mentor-Grade Cosmic Lotus Observatory 12x18 Poster Steampunk Study</t>
@@ -10984,9 +11528,21 @@
           <t>$34.99</t>
         </is>
       </c>
-      <c r="J159" t="inlineStr"/>
-      <c r="K159" t="inlineStr"/>
-      <c r="L159" t="inlineStr"/>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M159" t="b">
         <v>1</v>
       </c>
@@ -11018,7 +11574,7 @@
       </c>
       <c r="T159" t="inlineStr">
         <is>
-          <t>Etsy_Draft_Prepared</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -11048,8 +11604,16 @@
           <t>69f2a2aacaeb1241880b9f6b</t>
         </is>
       </c>
-      <c r="F160" t="inlineStr"/>
-      <c r="G160" t="inlineStr"/>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>406902691983</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902691983</t>
+        </is>
+      </c>
       <c r="H160" t="inlineStr">
         <is>
           <t>Astrolabe Chalice Relic Dark Academia Poster 12x18 Vintage Study Decor Wall</t>
@@ -11060,9 +11624,21 @@
           <t>$34.99</t>
         </is>
       </c>
-      <c r="J160" t="inlineStr"/>
-      <c r="K160" t="inlineStr"/>
-      <c r="L160" t="inlineStr"/>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M160" t="b">
         <v>0</v>
       </c>
@@ -11086,7 +11662,7 @@
       </c>
       <c r="T160" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -11116,8 +11692,16 @@
           <t>69f2a7d0e64c9f31b70f79cf</t>
         </is>
       </c>
-      <c r="F161" t="inlineStr"/>
-      <c r="G161" t="inlineStr"/>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>406902633400</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902633400</t>
+        </is>
+      </c>
       <c r="H161" t="inlineStr">
         <is>
           <t>Grimdark Alchemical Terrarium Withered Mandrake Root Chamber 5x7 Acrylic Block</t>
@@ -11128,9 +11712,21 @@
           <t>$89.99</t>
         </is>
       </c>
-      <c r="J161" t="inlineStr"/>
-      <c r="K161" t="inlineStr"/>
-      <c r="L161" t="inlineStr"/>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M161" t="b">
         <v>0</v>
       </c>
@@ -11154,7 +11750,7 @@
       </c>
       <c r="T161" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -11184,8 +11780,16 @@
           <t>69f2a8a5357398ded80f8faf</t>
         </is>
       </c>
-      <c r="F162" t="inlineStr"/>
-      <c r="G162" t="inlineStr"/>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>406902657898</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902657898</t>
+        </is>
+      </c>
       <c r="H162" t="inlineStr">
         <is>
           <t>Zen Aesthetic Ritual Bell Shrine 5x7 Acrylic Block for Meditation Desk Shelf</t>
@@ -11196,9 +11800,21 @@
           <t>$89.99</t>
         </is>
       </c>
-      <c r="J162" t="inlineStr"/>
-      <c r="K162" t="inlineStr"/>
-      <c r="L162" t="inlineStr"/>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M162" t="b">
         <v>1</v>
       </c>
@@ -11230,7 +11846,7 @@
       </c>
       <c r="T162" t="inlineStr">
         <is>
-          <t>Etsy_Draft_Prepared</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -11260,8 +11876,16 @@
           <t>69f2a9b45f78c14a7b0a7290</t>
         </is>
       </c>
-      <c r="F163" t="inlineStr"/>
-      <c r="G163" t="inlineStr"/>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>406902673249</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902673249</t>
+        </is>
+      </c>
       <c r="H163" t="inlineStr">
         <is>
           <t>Zen Pagoda Fragment Relic 5x7 Acrylic Print Floating Tower Decor Jade Framework</t>
@@ -11272,9 +11896,21 @@
           <t>$89.99</t>
         </is>
       </c>
-      <c r="J163" t="inlineStr"/>
-      <c r="K163" t="inlineStr"/>
-      <c r="L163" t="inlineStr"/>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M163" t="b">
         <v>0</v>
       </c>
@@ -11298,7 +11934,7 @@
       </c>
       <c r="T163" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -11328,8 +11964,16 @@
           <t>69f2b132cd8d04605103fdaa</t>
         </is>
       </c>
-      <c r="F164" t="inlineStr"/>
-      <c r="G164" t="inlineStr"/>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>406902882943</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902882943</t>
+        </is>
+      </c>
       <c r="H164" t="inlineStr">
         <is>
           <t>Orrery Lighthouse Beacon Dark Academia Poster 12x18 Vintage Astronomy Wall Art</t>
@@ -11340,9 +11984,21 @@
           <t>$34.99</t>
         </is>
       </c>
-      <c r="J164" t="inlineStr"/>
-      <c r="K164" t="inlineStr"/>
-      <c r="L164" t="inlineStr"/>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M164" t="b">
         <v>0</v>
       </c>
@@ -11366,7 +12022,7 @@
       </c>
       <c r="T164" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Has_View_Monitor</t>
         </is>
       </c>
     </row>
@@ -11396,8 +12052,16 @@
           <t>69f2b7ada7777da1971028d7</t>
         </is>
       </c>
-      <c r="F165" t="inlineStr"/>
-      <c r="G165" t="inlineStr"/>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>406902887127</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902887127</t>
+        </is>
+      </c>
       <c r="H165" t="inlineStr">
         <is>
           <t>Dark Academia Celestial Lotus Poster 12x18 Vintage Study Room Wall Art Decor</t>
@@ -11408,9 +12072,21 @@
           <t>$34.99</t>
         </is>
       </c>
-      <c r="J165" t="inlineStr"/>
-      <c r="K165" t="inlineStr"/>
-      <c r="L165" t="inlineStr"/>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M165" t="b">
         <v>1</v>
       </c>
@@ -11442,7 +12118,7 @@
       </c>
       <c r="T165" t="inlineStr">
         <is>
-          <t>Etsy_Draft_Prepared</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -11472,8 +12148,16 @@
           <t>69f2b9c3caeb1241880bae85</t>
         </is>
       </c>
-      <c r="F166" t="inlineStr"/>
-      <c r="G166" t="inlineStr"/>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>406902703464</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902703464</t>
+        </is>
+      </c>
       <c r="H166" t="inlineStr">
         <is>
           <t>Celestial Orrery Tree Bonsai Dark Academia 5x7 Acrylic Block Mentor-Grade Study</t>
@@ -11484,9 +12168,21 @@
           <t>$89.99</t>
         </is>
       </c>
-      <c r="J166" t="inlineStr"/>
-      <c r="K166" t="inlineStr"/>
-      <c r="L166" t="inlineStr"/>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M166" t="b">
         <v>0</v>
       </c>
@@ -11510,7 +12206,7 @@
       </c>
       <c r="T166" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -11540,8 +12236,16 @@
           <t>69f2bac6343d8ca093077dd8</t>
         </is>
       </c>
-      <c r="F167" t="inlineStr"/>
-      <c r="G167" t="inlineStr"/>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>406902885214</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902885214</t>
+        </is>
+      </c>
       <c r="H167" t="inlineStr">
         <is>
           <t>Grimdark Ritual Censer Thurible 5x7 Acrylic Block Dark Academia Mentor-Grade</t>
@@ -11552,9 +12256,21 @@
           <t>$89.99</t>
         </is>
       </c>
-      <c r="J167" t="inlineStr"/>
-      <c r="K167" t="inlineStr"/>
-      <c r="L167" t="inlineStr"/>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M167" t="b">
         <v>0</v>
       </c>
@@ -11578,7 +12294,7 @@
       </c>
       <c r="T167" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -11608,8 +12324,16 @@
           <t>69f2bbbc343d8ca093077e9a</t>
         </is>
       </c>
-      <c r="F168" t="inlineStr"/>
-      <c r="G168" t="inlineStr"/>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>406902888077</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902888077</t>
+        </is>
+      </c>
       <c r="H168" t="inlineStr">
         <is>
           <t>Zen Cyberpunk Koi Automaton 5x7 Acrylic Block - Meditative Desk Sculpture Shelf</t>
@@ -11620,9 +12344,21 @@
           <t>$89.99</t>
         </is>
       </c>
-      <c r="J168" t="inlineStr"/>
-      <c r="K168" t="inlineStr"/>
-      <c r="L168" t="inlineStr"/>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M168" t="b">
         <v>0</v>
       </c>
@@ -11646,7 +12382,7 @@
       </c>
       <c r="T168" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Has_View_Monitor</t>
         </is>
       </c>
     </row>
@@ -11676,8 +12412,16 @@
           <t>69f2c22e9b469f716d0ea954</t>
         </is>
       </c>
-      <c r="F169" t="inlineStr"/>
-      <c r="G169" t="inlineStr"/>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>406902893289</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902893289</t>
+        </is>
+      </c>
       <c r="H169" t="inlineStr">
         <is>
           <t>Zen Incense Vessel Constellation 5x7 Acrylic Block for Meditation Desk Shelf</t>
@@ -11688,9 +12432,21 @@
           <t>$89.99</t>
         </is>
       </c>
-      <c r="J169" t="inlineStr"/>
-      <c r="K169" t="inlineStr"/>
-      <c r="L169" t="inlineStr"/>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M169" t="b">
         <v>0</v>
       </c>
@@ -11714,7 +12470,7 @@
       </c>
       <c r="T169" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -11744,8 +12500,16 @@
           <t>69f2dc76cd8d046051041f06</t>
         </is>
       </c>
-      <c r="F170" t="inlineStr"/>
-      <c r="G170" t="inlineStr"/>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>406902890971</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902890971</t>
+        </is>
+      </c>
       <c r="H170" t="inlineStr">
         <is>
           <t>Zen Bonsai Wall Art Celestial Gate of Jade Mist 12x18 Poster Meditation Decor</t>
@@ -11756,9 +12520,21 @@
           <t>$34.99</t>
         </is>
       </c>
-      <c r="J170" t="inlineStr"/>
-      <c r="K170" t="inlineStr"/>
-      <c r="L170" t="inlineStr"/>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M170" t="b">
         <v>0</v>
       </c>
@@ -11782,7 +12558,7 @@
       </c>
       <c r="T170" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -11812,8 +12588,16 @@
           <t>69f2cf675f78c14a7b0a894c</t>
         </is>
       </c>
-      <c r="F171" t="inlineStr"/>
-      <c r="G171" t="inlineStr"/>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>406902897663</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902897663</t>
+        </is>
+      </c>
       <c r="H171" t="inlineStr">
         <is>
           <t>Dark Academia Phoenix Incense Burner 12x18 Poster Ritual Zen Decor Wall Study</t>
@@ -11824,9 +12608,21 @@
           <t>$34.99</t>
         </is>
       </c>
-      <c r="J171" t="inlineStr"/>
-      <c r="K171" t="inlineStr"/>
-      <c r="L171" t="inlineStr"/>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M171" t="b">
         <v>1</v>
       </c>
@@ -11858,7 +12654,7 @@
       </c>
       <c r="T171" t="inlineStr">
         <is>
-          <t>Etsy_Draft_Prepared</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -11952,8 +12748,16 @@
           <t>69f2d2a1c326d7da170c51b4</t>
         </is>
       </c>
-      <c r="F173" t="inlineStr"/>
-      <c r="G173" t="inlineStr"/>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>406902898909</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406902898909</t>
+        </is>
+      </c>
       <c r="H173" t="inlineStr">
         <is>
           <t>Zen Mentor-Grade Jade Phoenix Incense Altar 5x7 Acrylic Block for Meditation</t>
@@ -11964,9 +12768,21 @@
           <t>$89.99</t>
         </is>
       </c>
-      <c r="J173" t="inlineStr"/>
-      <c r="K173" t="inlineStr"/>
-      <c r="L173" t="inlineStr"/>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M173" t="b">
         <v>1</v>
       </c>
@@ -11998,7 +12814,7 @@
       </c>
       <c r="T173" t="inlineStr">
         <is>
-          <t>Etsy_Draft_Prepared</t>
+          <t>Published_Has_View_Monitor</t>
         </is>
       </c>
     </row>
@@ -12028,8 +12844,16 @@
           <t>69f2d3ab5f78c14a7b0a8b87</t>
         </is>
       </c>
-      <c r="F174" t="inlineStr"/>
-      <c r="G174" t="inlineStr"/>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>406903028253</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903028253</t>
+        </is>
+      </c>
       <c r="H174" t="inlineStr">
         <is>
           <t>Zen Aesthetic Sacred Lotus Meditation Bell 5x7 Acrylic Block for Altar Decor</t>
@@ -12040,9 +12864,21 @@
           <t>$89.99</t>
         </is>
       </c>
-      <c r="J174" t="inlineStr"/>
-      <c r="K174" t="inlineStr"/>
-      <c r="L174" t="inlineStr"/>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M174" t="b">
         <v>1</v>
       </c>
@@ -12074,7 +12910,7 @@
       </c>
       <c r="T174" t="inlineStr">
         <is>
-          <t>Etsy_Draft_Prepared</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -12104,8 +12940,16 @@
           <t>69f2d49b81039eb9ab0b583c</t>
         </is>
       </c>
-      <c r="F175" t="inlineStr"/>
-      <c r="G175" t="inlineStr"/>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>406903036452</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903036452</t>
+        </is>
+      </c>
       <c r="H175" t="inlineStr">
         <is>
           <t>Zen Celestial Bonsai Moon Garden 5x7 Acrylic Block for Serene Desk Decor Shelf</t>
@@ -12116,9 +12960,21 @@
           <t>$89.99</t>
         </is>
       </c>
-      <c r="J175" t="inlineStr"/>
-      <c r="K175" t="inlineStr"/>
-      <c r="L175" t="inlineStr"/>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M175" t="b">
         <v>0</v>
       </c>
@@ -12142,7 +12998,7 @@
       </c>
       <c r="T175" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -12172,8 +13028,16 @@
           <t>69f2dddb9577aaffd506bc32</t>
         </is>
       </c>
-      <c r="F176" t="inlineStr"/>
-      <c r="G176" t="inlineStr"/>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>406903026999</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903026999</t>
+        </is>
+      </c>
       <c r="H176" t="inlineStr">
         <is>
           <t>Zen Celestial Compass Poster 12x18 Wall Art Calm Study Decor Library Gift Room</t>
@@ -12184,9 +13048,21 @@
           <t>$34.99</t>
         </is>
       </c>
-      <c r="J176" t="inlineStr"/>
-      <c r="K176" t="inlineStr"/>
-      <c r="L176" t="inlineStr"/>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L176" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M176" t="b">
         <v>1</v>
       </c>
@@ -12218,7 +13094,7 @@
       </c>
       <c r="T176" t="inlineStr">
         <is>
-          <t>Etsy_Draft_Prepared</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -12248,8 +13124,16 @@
           <t>69f2db1a3c6616b960034a37</t>
         </is>
       </c>
-      <c r="F177" t="inlineStr"/>
-      <c r="G177" t="inlineStr"/>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>406903033377</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903033377</t>
+        </is>
+      </c>
       <c r="H177" t="inlineStr">
         <is>
           <t>Zen Phoenix Rebirth Vessel 12x18 Poster for Meditation Room Decor Wall Study</t>
@@ -12260,9 +13144,21 @@
           <t>$34.99</t>
         </is>
       </c>
-      <c r="J177" t="inlineStr"/>
-      <c r="K177" t="inlineStr"/>
-      <c r="L177" t="inlineStr"/>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M177" t="b">
         <v>0</v>
       </c>
@@ -12286,7 +13182,7 @@
       </c>
       <c r="T177" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -12316,8 +13212,16 @@
           <t>69f80ad2d3b9dc73b1051dbd</t>
         </is>
       </c>
-      <c r="F178" t="inlineStr"/>
-      <c r="G178" t="inlineStr"/>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>406903039716</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903039716</t>
+        </is>
+      </c>
       <c r="H178" t="inlineStr">
         <is>
           <t>Alchemical Star Flask Vessel 5x7 Acrylic Block Dark Academia Desk Decor Shelf</t>
@@ -12328,9 +13232,21 @@
           <t>$89.99</t>
         </is>
       </c>
-      <c r="J178" t="inlineStr"/>
-      <c r="K178" t="inlineStr"/>
-      <c r="L178" t="inlineStr"/>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M178" t="b">
         <v>1</v>
       </c>
@@ -12362,7 +13278,7 @@
       </c>
       <c r="T178" t="inlineStr">
         <is>
-          <t>Etsy_Draft_Prepared</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -12392,8 +13308,16 @@
           <t>69f2e4c77e3402ea470630eb</t>
         </is>
       </c>
-      <c r="F179" t="inlineStr"/>
-      <c r="G179" t="inlineStr"/>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>406903043482</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903043482</t>
+        </is>
+      </c>
       <c r="H179" t="inlineStr">
         <is>
           <t>Alchemist Divination Compass Grimdark 5x7 Acrylic Display Mentor-Grade Occult</t>
@@ -12404,9 +13328,21 @@
           <t>$89.99</t>
         </is>
       </c>
-      <c r="J179" t="inlineStr"/>
-      <c r="K179" t="inlineStr"/>
-      <c r="L179" t="inlineStr"/>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M179" t="b">
         <v>0</v>
       </c>
@@ -12430,7 +13366,7 @@
       </c>
       <c r="T179" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -12460,8 +13396,16 @@
           <t>69f80f8a83a8608fd80ec283</t>
         </is>
       </c>
-      <c r="F180" t="inlineStr"/>
-      <c r="G180" t="inlineStr"/>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>406903047385</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903047385</t>
+        </is>
+      </c>
       <c r="H180" t="inlineStr">
         <is>
           <t>Zen Bamboo Flute 5x7 Acrylic Block, Whispering Shakuhachi Meditation Art Gift</t>
@@ -12472,9 +13416,21 @@
           <t>$89.99</t>
         </is>
       </c>
-      <c r="J180" t="inlineStr"/>
-      <c r="K180" t="inlineStr"/>
-      <c r="L180" t="inlineStr"/>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M180" t="b">
         <v>0</v>
       </c>
@@ -12498,7 +13454,7 @@
       </c>
       <c r="T180" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -12528,8 +13484,16 @@
           <t>69f810485da263f75f049bf8</t>
         </is>
       </c>
-      <c r="F181" t="inlineStr"/>
-      <c r="G181" t="inlineStr"/>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>406903213858</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903213858</t>
+        </is>
+      </c>
       <c r="H181" t="inlineStr">
         <is>
           <t>Zen Lotus Seed Pod Vessel 5x7 Acrylic Block for Mindful Desk Decor Shelf Study</t>
@@ -12540,9 +13504,21 @@
           <t>$89.99</t>
         </is>
       </c>
-      <c r="J181" t="inlineStr"/>
-      <c r="K181" t="inlineStr"/>
-      <c r="L181" t="inlineStr"/>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M181" t="b">
         <v>0</v>
       </c>
@@ -12566,7 +13542,7 @@
       </c>
       <c r="T181" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -12596,8 +13572,16 @@
           <t>69f82b8aa1a4c45aad055063</t>
         </is>
       </c>
-      <c r="F182" t="inlineStr"/>
-      <c r="G182" t="inlineStr"/>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>406903249745</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903249745</t>
+        </is>
+      </c>
       <c r="H182" t="inlineStr">
         <is>
           <t>Gothic Lantern Soul Cage 5x7 Acrylic Block Grimdark Study Decor Crimson Flame</t>
@@ -12664,8 +13648,16 @@
           <t>69f82c8609f3b7302401cacf</t>
         </is>
       </c>
-      <c r="F183" t="inlineStr"/>
-      <c r="G183" t="inlineStr"/>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>406903250705</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903250705</t>
+        </is>
+      </c>
       <c r="H183" t="inlineStr">
         <is>
           <t>Grimdark Gothic Lantern 5x7 Acrylic Block Shadowbound Sentinel Beacon Dark Gift</t>
@@ -12732,8 +13724,16 @@
           <t>69f8388b25819cdf3d0538bc</t>
         </is>
       </c>
-      <c r="F184" t="inlineStr"/>
-      <c r="G184" t="inlineStr"/>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>406903251829</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903251829</t>
+        </is>
+      </c>
       <c r="H184" t="inlineStr">
         <is>
           <t>Gothic Necromancer Soul Reliquary 5x7 Acrylic Grimdark Artifact Decor Shelf</t>
@@ -12800,8 +13800,16 @@
           <t>69f83957ffbc831dea082e1a</t>
         </is>
       </c>
-      <c r="F185" t="inlineStr"/>
-      <c r="G185" t="inlineStr"/>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>406903252506</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903252506</t>
+        </is>
+      </c>
       <c r="H185" t="inlineStr">
         <is>
           <t>Gothic Grimdark Voidwalker Eternal Lamp 5x7 Acrylic Block Dark Decor Shelf Gift</t>
@@ -12868,8 +13876,16 @@
           <t>69f839eaf9374ed4f105a092</t>
         </is>
       </c>
-      <c r="F186" t="inlineStr"/>
-      <c r="G186" t="inlineStr"/>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>406903731967</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903731967</t>
+        </is>
+      </c>
       <c r="H186" t="inlineStr">
         <is>
           <t>Gothic Banshee Lantern Grimdark Art 5x7 Acrylic Premium Collectible Decor Shelf</t>
@@ -12936,8 +13952,16 @@
           <t>69f83a955da263f75f04c06a</t>
         </is>
       </c>
-      <c r="F187" t="inlineStr"/>
-      <c r="G187" t="inlineStr"/>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>406903746215</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903746215</t>
+        </is>
+      </c>
       <c r="H187" t="inlineStr">
         <is>
           <t>Gothic Grimdark Revenant Lantern 5x7 Acrylic Art Premium Decor Sapphire Glass</t>
@@ -13004,8 +14028,16 @@
           <t>69f83b5cf9374ed4f105a180</t>
         </is>
       </c>
-      <c r="F188" t="inlineStr"/>
-      <c r="G188" t="inlineStr"/>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>406903749989</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903749989</t>
+        </is>
+      </c>
       <c r="H188" t="inlineStr">
         <is>
           <t>Gothic Grimdark Lich Phylactery Lantern 5x7 Acrylic Print Dark Fantasy Home</t>
@@ -13072,8 +14104,16 @@
           <t>69f83c14ffbc831dea082fa3</t>
         </is>
       </c>
-      <c r="F189" t="inlineStr"/>
-      <c r="G189" t="inlineStr"/>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>406903756190</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903756190</t>
+        </is>
+      </c>
       <c r="H189" t="inlineStr">
         <is>
           <t>Gothic Wraith Warden Cursed Beacon 5x7 Acrylic Block Dark Fantasy Decor Shelf</t>
@@ -13140,8 +14180,16 @@
           <t>69f847b45da263f75f04cdbd</t>
         </is>
       </c>
-      <c r="F190" t="inlineStr"/>
-      <c r="G190" t="inlineStr"/>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>406903038850</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903038850</t>
+        </is>
+      </c>
       <c r="H190" t="inlineStr">
         <is>
           <t>Arcane Archway of Forbidden Chronicles Dark Academia 12x18 Poster Study Room</t>
@@ -13152,9 +14200,21 @@
           <t>$34.99</t>
         </is>
       </c>
-      <c r="J190" t="inlineStr"/>
-      <c r="K190" t="inlineStr"/>
-      <c r="L190" t="inlineStr"/>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L190" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M190" t="b">
         <v>0</v>
       </c>
@@ -13178,7 +14238,7 @@
       </c>
       <c r="T190" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -13208,8 +14268,16 @@
           <t>69f84864feed9979d10cd5ba</t>
         </is>
       </c>
-      <c r="F191" t="inlineStr"/>
-      <c r="G191" t="inlineStr"/>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>406903042690</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903042690</t>
+        </is>
+      </c>
       <c r="H191" t="inlineStr">
         <is>
           <t>Dark Academia Ethereal Torii Poster 12x18 Study Room Decor Scholarly Ascension</t>
@@ -13220,9 +14288,21 @@
           <t>$34.99</t>
         </is>
       </c>
-      <c r="J191" t="inlineStr"/>
-      <c r="K191" t="inlineStr"/>
-      <c r="L191" t="inlineStr"/>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L191" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M191" t="b">
         <v>1</v>
       </c>
@@ -13254,7 +14334,7 @@
       </c>
       <c r="T191" t="inlineStr">
         <is>
-          <t>Etsy_Draft_Prepared</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -13284,8 +14364,16 @@
           <t>69f84b3d5da263f75f04d1f7</t>
         </is>
       </c>
-      <c r="F192" t="inlineStr"/>
-      <c r="G192" t="inlineStr"/>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>406903046097</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903046097</t>
+        </is>
+      </c>
       <c r="H192" t="inlineStr">
         <is>
           <t>Dark Academia Mystic Threshold Infinite Knowledge Poster 12x18 Study Decor Wall</t>
@@ -13296,9 +14384,21 @@
           <t>$34.99</t>
         </is>
       </c>
-      <c r="J192" t="inlineStr"/>
-      <c r="K192" t="inlineStr"/>
-      <c r="L192" t="inlineStr"/>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M192" t="b">
         <v>1</v>
       </c>
@@ -13330,7 +14430,7 @@
       </c>
       <c r="T192" t="inlineStr">
         <is>
-          <t>Etsy_Draft_Prepared</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -13360,8 +14460,16 @@
           <t>69f8547125819cdf3d05522b</t>
         </is>
       </c>
-      <c r="F193" t="inlineStr"/>
-      <c r="G193" t="inlineStr"/>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>406903209258</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903209258</t>
+        </is>
+      </c>
       <c r="H193" t="inlineStr">
         <is>
           <t>Dark Academia Sanctum Gate of Preserved Wisdom 12x18 Poster Study Decor Wall</t>
@@ -13372,9 +14480,21 @@
           <t>$34.99</t>
         </is>
       </c>
-      <c r="J193" t="inlineStr"/>
-      <c r="K193" t="inlineStr"/>
-      <c r="L193" t="inlineStr"/>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M193" t="b">
         <v>0</v>
       </c>
@@ -13398,7 +14518,7 @@
       </c>
       <c r="T193" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -13428,8 +14548,16 @@
           <t>69f854ed09f3b7302401ed2e</t>
         </is>
       </c>
-      <c r="F194" t="inlineStr"/>
-      <c r="G194" t="inlineStr"/>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>406903249496</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903249496</t>
+        </is>
+      </c>
       <c r="H194" t="inlineStr">
         <is>
           <t>Dark Academia Hermetic Portal of Ancient Codices 12x18 Poster Study Decor Wall</t>
@@ -13496,8 +14624,16 @@
           <t>69f850b425819cdf3d054e10</t>
         </is>
       </c>
-      <c r="F195" t="inlineStr"/>
-      <c r="G195" t="inlineStr"/>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>406903250376</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903250376</t>
+        </is>
+      </c>
       <c r="H195" t="inlineStr">
         <is>
           <t>Dark Academia Celestial Archway Poster 12x18 Study Room Decor Timeless Tomes</t>
@@ -18966,8 +20102,76 @@
         </is>
       </c>
     </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0044-FIX1</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Printify_PublishExternalPending_Mockups3</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>69fbdfc9f60a24b6d1035f8b</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr"/>
+      <c r="G275" t="inlineStr"/>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>Zen Aesthetic Dragon Coil 4pc 6x6 Kiss-Cut Sticker Laptop Journal Water Bottle</t>
+        </is>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>$11.99</t>
+        </is>
+      </c>
+      <c r="J275" t="inlineStr"/>
+      <c r="K275" t="inlineStr"/>
+      <c r="L275" t="inlineStr"/>
+      <c r="M275" t="b">
+        <v>0</v>
+      </c>
+      <c r="N275" t="inlineStr"/>
+      <c r="O275" t="inlineStr"/>
+      <c r="P275" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0044_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="Q275" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0044_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="R275" t="b">
+        <v>1</v>
+      </c>
+      <c r="S275" t="b">
+        <v>1</v>
+      </c>
+      <c r="T275" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T274"/>
+  <autoFilter ref="A1:T275"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Restore cruise runtime and run Track B experiment
</commit_message>
<xml_diff>
--- a/Database/Unified_Listing_Registry.xlsx
+++ b/Database/Unified_Listing_Registry.xlsx
@@ -5756,7 +5756,7 @@
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
         <is>
-          <t>Celestial Koi Constellation 4pc 6x6 Kiss-Cut Sticker Zen Aesthetic Laptop Vinyl</t>
+          <t>Deep Work Sticker Set Celestial Koi Constellation 4pc 6x6 Vinyl Laptop Journal</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -5786,7 +5786,7 @@
         <v>1</v>
       </c>
       <c r="S73" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T73" t="inlineStr">
         <is>
@@ -5824,7 +5824,7 @@
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
-          <t>Sacred Singing Bowl Mindful Zen 4pc 6x6 Vinyl Sticker Yoga Minimalist Gift Gift</t>
+          <t>Book Nook Laptop Decals Sacred Singing Bowl Yoga Minimalist 4pc 6x6 Kiss-Cut</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -5854,7 +5854,7 @@
         <v>1</v>
       </c>
       <c r="S74" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T74" t="inlineStr">
         <is>
@@ -5892,7 +5892,7 @@
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Minimal Zen Bamboo Pagoda Relic 4pc 6x6 Sticker Sheet Serene Mindful Clean Gift</t>
+          <t>Deep Work Sticker Set Bamboo Pagoda Relic Serene Clean 4pc 6x6 Vinyl Laptop</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -5922,7 +5922,7 @@
         <v>1</v>
       </c>
       <c r="S75" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T75" t="inlineStr">
         <is>
@@ -5960,7 +5960,7 @@
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
-          <t>Mindful Zen Dragon Pearl Talisman 4pc 6x6 Vinyl Sticker Laptop Journal Gift</t>
+          <t>Book Nook Laptop Decals Dragon Pearl Talisman 4pc 6x6 Kiss-Cut Sticker Set Gift</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -5990,7 +5990,7 @@
         <v>1</v>
       </c>
       <c r="S76" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T76" t="inlineStr">
         <is>
@@ -6028,7 +6028,7 @@
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Moonlit Mountain Shrine Mindful Zen 4pc 6x6 Vinyl Sticker Yoga Minimalist Gift</t>
+          <t>Deep Work Sticker Set Moonlit Mountain Shrine Yoga Minimalist 4pc 6x6 Vinyl</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -6058,7 +6058,7 @@
         <v>1</v>
       </c>
       <c r="S77" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T77" t="inlineStr">
         <is>
@@ -6288,7 +6288,7 @@
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Celestial Koi Ascension Minimal Zen 4pc 6x6 Kiss-Cut Vinyl Desk Collector Decor</t>
+          <t>Deep Work Sticker Set Celestial Koi Ascension Collector 4pc 6x6 Vinyl Laptop</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -6318,7 +6318,7 @@
         <v>1</v>
       </c>
       <c r="S81" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T81" t="inlineStr">
         <is>
@@ -6420,7 +6420,7 @@
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
         <is>
-          <t>Phoenix Wing Fragment 4pc 6x6 Kiss-Cut Sticker Zen Aesthetic Laptop Journal</t>
+          <t>Deep Work Sticker Set Phoenix Wing Fragment 4pc 6x6 Vinyl Laptop Journal Decor</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -6450,7 +6450,7 @@
         <v>1</v>
       </c>
       <c r="S83" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T83" t="inlineStr">
         <is>
@@ -12796,7 +12796,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>Zen Mentor-Grade Jade Phoenix Incense Altar 5x7 Acrylic Block for Meditation</t>
+          <t>Meditation Room Jade Relic Phoenix 5x7 Acrylic Block Shelf Decor Gift Study</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -12846,7 +12846,7 @@
         <v>1</v>
       </c>
       <c r="S173" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T173" t="inlineStr">
         <is>
@@ -12892,7 +12892,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>Quiet Luxury Shelf Decor Sacred Lotus Meditation Bell for 5x7 Acrylic Photo</t>
+          <t>Meditation Room Jade Relic Quiet Luxury 5x7 Acrylic Block Shelf Decor Gift Wall</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -13356,7 +13356,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>Gallery Desk Art Alchemist Divination Compass Occult 5x7 Acrylic Photo Block</t>
+          <t>Dark Study Smoky Jade Alchemist Divination Compass 5x7 Acrylic Block Shelf Gift</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -15216,7 +15216,7 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>Soulbound Harbinger Torch Grimdark Gothic Lantern 5x7 Acrylic Print Dark Decor</t>
+          <t>Quiet Luxury Jade Relic Soulbound 5x7 Acrylic Block Shelf Decor Gift Study Wall</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -15246,7 +15246,7 @@
         <v>1</v>
       </c>
       <c r="S201" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T201" t="inlineStr">
         <is>
@@ -15356,8 +15356,16 @@
           <t>69f86a3d25819cdf3d0563b6</t>
         </is>
       </c>
-      <c r="F203" t="inlineStr"/>
-      <c r="G203" t="inlineStr"/>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>406909215172</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909215172</t>
+        </is>
+      </c>
       <c r="H203" t="inlineStr">
         <is>
           <t>Gothic Grimdark Shadowpriest Ritual Vessel 5x7 Acrylic Decor Indigo Flame Shelf</t>
@@ -15424,8 +15432,16 @@
           <t>69f86b8e83a8608fd80f1341</t>
         </is>
       </c>
-      <c r="F204" t="inlineStr"/>
-      <c r="G204" t="inlineStr"/>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>406909219066</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909219066</t>
+        </is>
+      </c>
       <c r="H204" t="inlineStr">
         <is>
           <t>Grimdark Aesthetic Dreadlord Beacon Lantern 5x7 Acrylic Block Dark Decor Shelf</t>
@@ -15492,8 +15508,16 @@
           <t>69f86d3709f3b730240200b7</t>
         </is>
       </c>
-      <c r="F205" t="inlineStr"/>
-      <c r="G205" t="inlineStr"/>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>406909222169</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909222169</t>
+        </is>
+      </c>
       <c r="H205" t="inlineStr">
         <is>
           <t>Sepulcher Guardian's Flame Grimdark Gothic Lantern 5x7 Acrylic Art Dark Shelf</t>
@@ -15560,11 +15584,19 @@
           <t>69f86f6c2810b52a940a4161</t>
         </is>
       </c>
-      <c r="F206" t="inlineStr"/>
-      <c r="G206" t="inlineStr"/>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>406909223875</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909223875</t>
+        </is>
+      </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>Abyssal Watcher Eternal Eye Grimdark Gothic Acrylic 5x7 Spirit Beacon Artifact</t>
+          <t>Quiet Luxury Jade Relic Abyssal 5x7 Acrylic Block Shelf Decor Gift Study Wall</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
@@ -15594,7 +15626,7 @@
         <v>1</v>
       </c>
       <c r="S206" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T206" t="inlineStr">
         <is>
@@ -15628,8 +15660,16 @@
           <t>69f8807a011b67ecf80761ae</t>
         </is>
       </c>
-      <c r="F207" t="inlineStr"/>
-      <c r="G207" t="inlineStr"/>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>406909225478</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909225478</t>
+        </is>
+      </c>
       <c r="H207" t="inlineStr">
         <is>
           <t>Emerald Despair Lantern Grimdark Gothic Ironwork 5x7 Acrylic Block Dark Fantasy</t>
@@ -15696,8 +15736,16 @@
           <t>69f8818abe136844f0003e48</t>
         </is>
       </c>
-      <c r="F208" t="inlineStr"/>
-      <c r="G208" t="inlineStr"/>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>406909226531</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909226531</t>
+        </is>
+      </c>
       <c r="H208" t="inlineStr">
         <is>
           <t>Violet Torment Lantern 5x7 Acrylic Grimdark Gothic Decor for Dark Fantasy Study</t>
@@ -15764,8 +15812,16 @@
           <t>69f882a1be136844f0003eed</t>
         </is>
       </c>
-      <c r="F209" t="inlineStr"/>
-      <c r="G209" t="inlineStr"/>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>406909228840</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909228840</t>
+        </is>
+      </c>
       <c r="H209" t="inlineStr">
         <is>
           <t>Azure Suffering Lantern 5x7 Acrylic Grimdark Gothic Wall Art Decor Shelf Study</t>
@@ -15832,8 +15888,16 @@
           <t>69f8836c5da263f75f04fad5</t>
         </is>
       </c>
-      <c r="F210" t="inlineStr"/>
-      <c r="G210" t="inlineStr"/>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>406909231370</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909231370</t>
+        </is>
+      </c>
       <c r="H210" t="inlineStr">
         <is>
           <t>Grimdark Obsidian Wrath Lantern 5x7 Acrylic Block Dark Fantasy Desk Art Shelf</t>
@@ -15900,8 +15964,16 @@
           <t>69f883f3be136844f0003ff9</t>
         </is>
       </c>
-      <c r="F211" t="inlineStr"/>
-      <c r="G211" t="inlineStr"/>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>406909232068</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909232068</t>
+        </is>
+      </c>
       <c r="H211" t="inlineStr">
         <is>
           <t>Amber Anguish Lantern Grimdark Aesthetic 5x7 Acrylic Art Decor Shelf Study Gift</t>
@@ -15968,8 +16040,16 @@
           <t>69f88472ffbc831dea086941</t>
         </is>
       </c>
-      <c r="F212" t="inlineStr"/>
-      <c r="G212" t="inlineStr"/>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>406909232951</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909232951</t>
+        </is>
+      </c>
       <c r="H212" t="inlineStr">
         <is>
           <t>Frost Agony Lantern Grimdark Ice Spirit 5x7 Acrylic Art Gothic Decor Shelf Gift</t>
@@ -16036,11 +16116,19 @@
           <t>69f884ed83a8608fd80f239c</t>
         </is>
       </c>
-      <c r="F213" t="inlineStr"/>
-      <c r="G213" t="inlineStr"/>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>406909233684</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909233684</t>
+        </is>
+      </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>Magenta Malice Lantern Grimdark Mentor-Grade 5x7 Acrylic Decor Dark Fantasy</t>
+          <t>Quiet Luxury Jade Relic Magenta 5x7 Acrylic Block Shelf Decor Gift Study Wall</t>
         </is>
       </c>
       <c r="I213" t="inlineStr">
@@ -16070,7 +16158,7 @@
         <v>1</v>
       </c>
       <c r="S213" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T213" t="inlineStr">
         <is>
@@ -16104,8 +16192,16 @@
           <t>69f88562be136844f00040a3</t>
         </is>
       </c>
-      <c r="F214" t="inlineStr"/>
-      <c r="G214" t="inlineStr"/>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>406909234435</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909234435</t>
+        </is>
+      </c>
       <c r="H214" t="inlineStr">
         <is>
           <t>Gothic Obsidian Shrine Soul Lantern 5x7 Acrylic Grimdark Artifact Display Shelf</t>
@@ -16172,8 +16268,16 @@
           <t>69f886005da263f75f04fc9d</t>
         </is>
       </c>
-      <c r="F215" t="inlineStr"/>
-      <c r="G215" t="inlineStr"/>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>406909235356</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909235356</t>
+        </is>
+      </c>
       <c r="H215" t="inlineStr">
         <is>
           <t>Spectral Temple Soul Lantern Grimdark Mentor-Grade 5x7 Acrylic Art Collectible</t>
@@ -16240,8 +16344,16 @@
           <t>69f88ee825819cdf3d057c87</t>
         </is>
       </c>
-      <c r="F216" t="inlineStr"/>
-      <c r="G216" t="inlineStr"/>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>406909236640</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909236640</t>
+        </is>
+      </c>
       <c r="H216" t="inlineStr">
         <is>
           <t>Midnight Sanctuary Soul Lantern Grimdark 5x7 Acrylic Collectible Display Shelf</t>
@@ -16308,8 +16420,16 @@
           <t>69f88fd4feed9979d10d0ce7</t>
         </is>
       </c>
-      <c r="F217" t="inlineStr"/>
-      <c r="G217" t="inlineStr"/>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>406909238227</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909238227</t>
+        </is>
+      </c>
       <c r="H217" t="inlineStr">
         <is>
           <t>Grimdark Amber Monastery Soul Lantern 5x7 Acrylic Art Gothic Decor Golden Flame</t>
@@ -16376,11 +16496,19 @@
           <t>69f8904bc1f268dee601c34f</t>
         </is>
       </c>
-      <c r="F218" t="inlineStr"/>
-      <c r="G218" t="inlineStr"/>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>406909240724</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909240724</t>
+        </is>
+      </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>Grimdark Ethereal Archway Soul Lantern 5x7 Acrylic Display Gothic Artifact Gift</t>
+          <t>Dark Study Smoky Jade Ethereal Archway Soul 5x7 Acrylic Block Shelf Decor Gift</t>
         </is>
       </c>
       <c r="I218" t="inlineStr">
@@ -16410,7 +16538,7 @@
         <v>1</v>
       </c>
       <c r="S218" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T218" t="inlineStr">
         <is>
@@ -16444,8 +16572,16 @@
           <t>69f890b8c1f268dee601c394</t>
         </is>
       </c>
-      <c r="F219" t="inlineStr"/>
-      <c r="G219" t="inlineStr"/>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>406909242546</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909242546</t>
+        </is>
+      </c>
       <c r="H219" t="inlineStr">
         <is>
           <t>Emerald Sanctum Soul Lantern Grimdark Art 5x7 Acrylic Mentor-Grade Collectible</t>
@@ -16512,8 +16648,16 @@
           <t>69f89116b051b8a0e90b9662</t>
         </is>
       </c>
-      <c r="F220" t="inlineStr"/>
-      <c r="G220" t="inlineStr"/>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>406909243824</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909243824</t>
+        </is>
+      </c>
       <c r="H220" t="inlineStr">
         <is>
           <t>Twilight Portal Soul Lantern Grimdark 5x7 Acrylic Art Gothic Decor Purple Flame</t>
@@ -16580,8 +16724,16 @@
           <t>69f8918925819cdf3d057e2d</t>
         </is>
       </c>
-      <c r="F221" t="inlineStr"/>
-      <c r="G221" t="inlineStr"/>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>406909244688</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909244688</t>
+        </is>
+      </c>
       <c r="H221" t="inlineStr">
         <is>
           <t>Gothic Frost Cathedral Soul Lantern 5x7 Acrylic Display Grimdark Artifact Shelf</t>
@@ -16648,8 +16800,16 @@
           <t>69f892035da263f75f05059e</t>
         </is>
       </c>
-      <c r="F222" t="inlineStr"/>
-      <c r="G222" t="inlineStr"/>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>406909247161</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909247161</t>
+        </is>
+      </c>
       <c r="H222" t="inlineStr">
         <is>
           <t>Gothic Onyx Shrine Soul Lantern 5x7 Acrylic Display Grimdark Collectible Shelf</t>
@@ -16708,7 +16868,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups4</t>
+          <t>Printify_Published_Mockups4</t>
         </is>
       </c>
       <c r="E223" t="inlineStr">
@@ -16716,11 +16876,19 @@
           <t>69f8928b25819cdf3d057ef7</t>
         </is>
       </c>
-      <c r="F223" t="inlineStr"/>
-      <c r="G223" t="inlineStr"/>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>406910074365</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406910074365</t>
+        </is>
+      </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>Rose Quartz Chapel Soul Lantern Grimdark 5x7 Acrylic Art Gothic Collectible</t>
+          <t>Collector Shelf Smoky Jade Quiet Luxury 5x7 Acrylic Block Shelf Decor Gift Wall</t>
         </is>
       </c>
       <c r="I223" t="inlineStr">
@@ -16750,11 +16918,11 @@
         <v>1</v>
       </c>
       <c r="S223" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T223" t="inlineStr">
         <is>
-          <t>Stable_Draft_Publish_When_Scheduled</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -16776,7 +16944,7 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups4</t>
+          <t>Printify_Published_Mockups4</t>
         </is>
       </c>
       <c r="E224" t="inlineStr">
@@ -16784,11 +16952,19 @@
           <t>69f8931cb051b8a0e90b97c7</t>
         </is>
       </c>
-      <c r="F224" t="inlineStr"/>
-      <c r="G224" t="inlineStr"/>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>406910075457</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406910075457</t>
+        </is>
+      </c>
       <c r="H224" t="inlineStr">
         <is>
-          <t>Sapphire Temple Soul Lantern Grimdark 5x7 Acrylic Display Gothic Artifact Shelf</t>
+          <t>Smoky Jade Gothic Object Sapphire Temple Soul Lantern Artifact 5x7 Acrylic Gift</t>
         </is>
       </c>
       <c r="I224" t="inlineStr">
@@ -16818,11 +16994,11 @@
         <v>1</v>
       </c>
       <c r="S224" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T224" t="inlineStr">
         <is>
-          <t>Stable_Draft_Publish_When_Scheduled</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -16844,7 +17020,7 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups4</t>
+          <t>Printify_Published_Mockups4</t>
         </is>
       </c>
       <c r="E225" t="inlineStr">
@@ -16852,11 +17028,19 @@
           <t>69f8937bbe136844f0004b36</t>
         </is>
       </c>
-      <c r="F225" t="inlineStr"/>
-      <c r="G225" t="inlineStr"/>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>406910076542</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406910076542</t>
+        </is>
+      </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t>Silver Moon Gate Soul Lantern Grimdark 5x7 Acrylic Art Gothic Mentor-Grade Gift</t>
+          <t>Smoky Jade Gothic Object Silver Moon Gate Soul Lantern 5x7 Acrylic Display Gift</t>
         </is>
       </c>
       <c r="I225" t="inlineStr">
@@ -16886,11 +17070,11 @@
         <v>1</v>
       </c>
       <c r="S225" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T225" t="inlineStr">
         <is>
-          <t>Stable_Draft_Publish_When_Scheduled</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -16920,8 +17104,16 @@
           <t>69f89a94c1f268dee601cb9d</t>
         </is>
       </c>
-      <c r="F226" t="inlineStr"/>
-      <c r="G226" t="inlineStr"/>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>406903730229</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903730229</t>
+        </is>
+      </c>
       <c r="H226" t="inlineStr">
         <is>
           <t>Dark Academia Poster 12x18 Magister Torii Study Decor Scholarly Gift Wall Room</t>
@@ -16988,11 +17180,19 @@
           <t>69f89b9ca70f06579a00a708</t>
         </is>
       </c>
-      <c r="F227" t="inlineStr"/>
-      <c r="G227" t="inlineStr"/>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>406903744471</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903744471</t>
+        </is>
+      </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>Dark Academia Archivist Gateway Poster 12x18 Vintage Study Room Decor Wall Gift</t>
+          <t>Reading Nook Smoky Jade Wall Art Archivist 12x18 Matte Poster Apartment Decor</t>
         </is>
       </c>
       <c r="I227" t="inlineStr">
@@ -17022,7 +17222,7 @@
         <v>1</v>
       </c>
       <c r="S227" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T227" t="inlineStr">
         <is>
@@ -17056,8 +17256,16 @@
           <t>69f89c6f09f3b730240221b8</t>
         </is>
       </c>
-      <c r="F228" t="inlineStr"/>
-      <c r="G228" t="inlineStr"/>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>406903748661</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903748661</t>
+        </is>
+      </c>
       <c r="H228" t="inlineStr">
         <is>
           <t>Dark Academia Mentor Threshold Poster 12x18 Intellectual Study Room Decor Wall</t>
@@ -17124,8 +17332,16 @@
           <t>69f89da69f68ab7cf001f531</t>
         </is>
       </c>
-      <c r="F229" t="inlineStr"/>
-      <c r="G229" t="inlineStr"/>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>406903754696</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903754696</t>
+        </is>
+      </c>
       <c r="H229" t="inlineStr">
         <is>
           <t>Dark Academia Celestial Chronometer Archive Sphere 12x18 Poster Study Decor</t>
@@ -17200,8 +17416,16 @@
           <t>69f89eac011b67ecf8077844</t>
         </is>
       </c>
-      <c r="F230" t="inlineStr"/>
-      <c r="G230" t="inlineStr"/>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>406903758348</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903758348</t>
+        </is>
+      </c>
       <c r="H230" t="inlineStr">
         <is>
           <t>Dark Academia Temporal Reliquary Bell Jar 12x18 Poster Study Decor Wall Library</t>
@@ -17268,8 +17492,16 @@
           <t>69f89fda2592a8ad8e0f2e79</t>
         </is>
       </c>
-      <c r="F231" t="inlineStr"/>
-      <c r="G231" t="inlineStr"/>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>406909147173</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909147173</t>
+        </is>
+      </c>
       <c r="H231" t="inlineStr">
         <is>
           <t>Hermetic Knowledge Lantern Dark Academia Poster 12x18 Library Decor Wall Study</t>
@@ -17336,8 +17568,16 @@
           <t>69f8a454c1f268dee601d3ad</t>
         </is>
       </c>
-      <c r="F232" t="inlineStr"/>
-      <c r="G232" t="inlineStr"/>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>406909150037</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909150037</t>
+        </is>
+      </c>
       <c r="H232" t="inlineStr">
         <is>
           <t>Dark Academia Industrial Library Pressure Chamber Poster 12x18 Vintage Decor</t>
@@ -17404,8 +17644,16 @@
           <t>69f903dec1f268dee601f679</t>
         </is>
       </c>
-      <c r="F233" t="inlineStr"/>
-      <c r="G233" t="inlineStr"/>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>406909153504</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909153504</t>
+        </is>
+      </c>
       <c r="H233" t="inlineStr">
         <is>
           <t>Dark Academia Chrono-Codex Terrarium 12x18 Poster Library Decor Wall Study Gift</t>
@@ -17472,8 +17720,16 @@
           <t>69f904df97d964f736006a48</t>
         </is>
       </c>
-      <c r="F234" t="inlineStr"/>
-      <c r="G234" t="inlineStr"/>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>406909164941</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909164941</t>
+        </is>
+      </c>
       <c r="H234" t="inlineStr">
         <is>
           <t>Dark Academia Apothecary Cylinder 12x18 Poster Vintage Study Decor Wall Library</t>
@@ -17548,8 +17804,16 @@
           <t>69f90607feed9979d10d40e7</t>
         </is>
       </c>
-      <c r="F235" t="inlineStr"/>
-      <c r="G235" t="inlineStr"/>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>406909216787</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909216787</t>
+        </is>
+      </c>
       <c r="H235" t="inlineStr">
         <is>
           <t>Dark Academia Astrolabe Dome Poster 12x18 Vintage Study Room Decor Wall Library</t>
@@ -17624,8 +17888,16 @@
           <t>69f907b49f68ab7cf0022003</t>
         </is>
       </c>
-      <c r="F236" t="inlineStr"/>
-      <c r="G236" t="inlineStr"/>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>406909220927</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909220927</t>
+        </is>
+      </c>
       <c r="H236" t="inlineStr">
         <is>
           <t>Dark Academia Alchemist Retort Library Poster 12x18 Study Decor Wall Gift Room</t>
@@ -17700,8 +17972,16 @@
           <t>69f90c957f4b346c8a0c603f</t>
         </is>
       </c>
-      <c r="F237" t="inlineStr"/>
-      <c r="G237" t="inlineStr"/>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>406909264998</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909264998</t>
+        </is>
+      </c>
       <c r="H237" t="inlineStr">
         <is>
           <t>Dark Academia Grimoire Preservation Capsule 12x18 Poster Study Decor Wall Gift</t>
@@ -17768,8 +18048,16 @@
           <t>69fba23409770f1d9306b86d</t>
         </is>
       </c>
-      <c r="F238" t="inlineStr"/>
-      <c r="G238" t="inlineStr"/>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>406909266188</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909266188</t>
+        </is>
+      </c>
       <c r="H238" t="inlineStr">
         <is>
           <t>Dark Academia Botanical Codex Conservatory Poster 12x18 Study Decor Wall Gift</t>
@@ -17836,8 +18124,16 @@
           <t>69fba266489d5635ab0e6504</t>
         </is>
       </c>
-      <c r="F239" t="inlineStr"/>
-      <c r="G239" t="inlineStr"/>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>406909268494</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909268494</t>
+        </is>
+      </c>
       <c r="H239" t="inlineStr">
         <is>
           <t>Dark Academia Observatory Archive Prism 12x18 Poster Study Room Decor Wall Gift</t>
@@ -17904,8 +18200,16 @@
           <t>69fba28a6d07bd21600e1684</t>
         </is>
       </c>
-      <c r="F240" t="inlineStr"/>
-      <c r="G240" t="inlineStr"/>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>406909269321</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909269321</t>
+        </is>
+      </c>
       <c r="H240" t="inlineStr">
         <is>
           <t>Dark Academia Philosophical Theorem Reliquary Poster 12x18 Study Decor Wall</t>
@@ -17972,8 +18276,16 @@
           <t>69fbbffef60a24b6d1034e4d</t>
         </is>
       </c>
-      <c r="F241" t="inlineStr"/>
-      <c r="G241" t="inlineStr"/>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>406909467980</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909467980</t>
+        </is>
+      </c>
       <c r="H241" t="inlineStr">
         <is>
           <t>Dark Academia Nautical Archive Barometer 12x18 Poster Study Decor Wall Library</t>
@@ -18108,8 +18420,16 @@
           <t>69fb7e754ce71ea8ae0c7af1</t>
         </is>
       </c>
-      <c r="F243" t="inlineStr"/>
-      <c r="G243" t="inlineStr"/>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>406909061109</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909061109</t>
+        </is>
+      </c>
       <c r="H243" t="inlineStr">
         <is>
           <t>Forbidden Grimoire Lock 4pc 6x6 Kiss-Cut Sticker Dark Academia Laptop Journal</t>
@@ -18176,8 +18496,16 @@
           <t>69fb804bff28e7d4030aa67d</t>
         </is>
       </c>
-      <c r="F244" t="inlineStr"/>
-      <c r="G244" t="inlineStr"/>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>406909095974</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909095974</t>
+        </is>
+      </c>
       <c r="H244" t="inlineStr">
         <is>
           <t>4pc Sticker Set Botanical Terrarium Lantern Vinyl Decals Laptop Bottle Dark</t>
@@ -18244,8 +18572,16 @@
           <t>69fb819d4c6544084c0f8370</t>
         </is>
       </c>
-      <c r="F245" t="inlineStr"/>
-      <c r="G245" t="inlineStr"/>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>406909097469</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909097469</t>
+        </is>
+      </c>
       <c r="H245" t="inlineStr">
         <is>
           <t>4pc Kiss-Cut Sticker Set Astrolabe Navigation Instrument Laptop Journal Bottle</t>
@@ -18312,8 +18648,16 @@
           <t>69fb82e64c6544084c0f83d5</t>
         </is>
       </c>
-      <c r="F246" t="inlineStr"/>
-      <c r="G246" t="inlineStr"/>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>406909100892</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909100892</t>
+        </is>
+      </c>
       <c r="H246" t="inlineStr">
         <is>
           <t>Ritual Incense Censer Gothic Academia 4pc 6x6 Vinyl Sticker Reader Writer Decor</t>
@@ -18380,8 +18724,16 @@
           <t>69fb868dc5114ecf420d2b93</t>
         </is>
       </c>
-      <c r="F247" t="inlineStr"/>
-      <c r="G247" t="inlineStr"/>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>406909114799</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909114799</t>
+        </is>
+      </c>
       <c r="H247" t="inlineStr">
         <is>
           <t>4pc Sticker Set Gothic Academia Cathedral Fragment Vinyl Decals Laptop Bottle</t>
@@ -18448,8 +18800,16 @@
           <t>69fb8749a7afceb9f70f1956</t>
         </is>
       </c>
-      <c r="F248" t="inlineStr"/>
-      <c r="G248" t="inlineStr"/>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>406909116716</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909116716</t>
+        </is>
+      </c>
       <c r="H248" t="inlineStr">
         <is>
           <t>Vintage Academia Compass Rose Talisman 4pc 6x6 Sticker Sheet Literary Cozy Gift</t>
@@ -18516,8 +18876,16 @@
           <t>69fb87aca7afceb9f70f1982</t>
         </is>
       </c>
-      <c r="F249" t="inlineStr"/>
-      <c r="G249" t="inlineStr"/>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>406909118000</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909118000</t>
+        </is>
+      </c>
       <c r="H249" t="inlineStr">
         <is>
           <t>Apothecary Poison Vial Vintage Academia 4pc 6x6 Kiss-Cut Vinyl Desk Collector</t>
@@ -18584,8 +18952,16 @@
           <t>69fb87efc5114ecf420d2c5a</t>
         </is>
       </c>
-      <c r="F250" t="inlineStr"/>
-      <c r="G250" t="inlineStr"/>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>406909119544</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909119544</t>
+        </is>
+      </c>
       <c r="H250" t="inlineStr">
         <is>
           <t>4pc Vinyl Sticker Set Microscope Observation Device Laptop Bottle Journal Dark</t>
@@ -18652,8 +19028,16 @@
           <t>69fb8805ee663532c8017f4f</t>
         </is>
       </c>
-      <c r="F251" t="inlineStr"/>
-      <c r="G251" t="inlineStr"/>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>406909121336</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909121336</t>
+        </is>
+      </c>
       <c r="H251" t="inlineStr">
         <is>
           <t>4pc Sticker Set Skeleton Key Portal Vinyl Decals Laptop Bottle Dark Academia</t>
@@ -18720,8 +19104,16 @@
           <t>69fb8811e5402c478e03108f</t>
         </is>
       </c>
-      <c r="F252" t="inlineStr"/>
-      <c r="G252" t="inlineStr"/>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>406909122790</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909122790</t>
+        </is>
+      </c>
       <c r="H252" t="inlineStr">
         <is>
           <t>4pc Kiss-Cut Sticker Set Gothic Academia Prism Light Refractor Laptop Journal</t>
@@ -18788,8 +19180,16 @@
           <t>69fb881f2b1da07362014876</t>
         </is>
       </c>
-      <c r="F253" t="inlineStr"/>
-      <c r="G253" t="inlineStr"/>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>406909124585</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909124585</t>
+        </is>
+      </c>
       <c r="H253" t="inlineStr">
         <is>
           <t>4pc Sticker Set Mindful Zen Koi Pond Vinyl Decals Laptop Bottle Zen Aesthetic</t>
@@ -18856,8 +19256,16 @@
           <t>69fb882c54fd3fbacf051371</t>
         </is>
       </c>
-      <c r="F254" t="inlineStr"/>
-      <c r="G254" t="inlineStr"/>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>406909125700</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909125700</t>
+        </is>
+      </c>
       <c r="H254" t="inlineStr">
         <is>
           <t>Minimal Zen Bonsai Tree of Serenity 4pc 6x6 Sticker Sheet Serene Mindful Clean</t>
@@ -18924,8 +19332,16 @@
           <t>69fb883cce0d8cb5570fa7cc</t>
         </is>
       </c>
-      <c r="F255" t="inlineStr"/>
-      <c r="G255" t="inlineStr"/>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>406909126789</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909126789</t>
+        </is>
+      </c>
       <c r="H255" t="inlineStr">
         <is>
           <t>Lotus Mandala Mindful Zen 4pc 6x6 Vinyl Sticker Yoga Minimalist Gift Gift Decor</t>
@@ -18992,8 +19408,16 @@
           <t>69fb8849e5402c478e0310af</t>
         </is>
       </c>
-      <c r="F256" t="inlineStr"/>
-      <c r="G256" t="inlineStr"/>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>406909127704</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909127704</t>
+        </is>
+      </c>
       <c r="H256" t="inlineStr">
         <is>
           <t>4pc Sticker Set Stone Guardian Lion Mindful Zen Vinyl Decals Laptop Bottle Zen</t>
@@ -19060,8 +19484,16 @@
           <t>69fbae614c6544084c0f95ec</t>
         </is>
       </c>
-      <c r="F257" t="inlineStr"/>
-      <c r="G257" t="inlineStr"/>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>406909342825</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909342825</t>
+        </is>
+      </c>
       <c r="H257" t="inlineStr">
         <is>
           <t>Bamboo Forest Minimal Zen 4pc 6x6 Kiss-Cut Vinyl Desk Collector Decor Misty Art</t>
@@ -19128,8 +19560,16 @@
           <t>69fbae7da7afceb9f70f2982</t>
         </is>
       </c>
-      <c r="F258" t="inlineStr"/>
-      <c r="G258" t="inlineStr"/>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>406909344491</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909344491</t>
+        </is>
+      </c>
       <c r="H258" t="inlineStr">
         <is>
           <t>4pc Sticker Set Cherry Blossom Branch Vinyl Decals Laptop Bottle Zen Aesthetic</t>
@@ -19196,8 +19636,16 @@
           <t>69fbae974c6544084c0f9610</t>
         </is>
       </c>
-      <c r="F259" t="inlineStr"/>
-      <c r="G259" t="inlineStr"/>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>406909345291</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909345291</t>
+        </is>
+      </c>
       <c r="H259" t="inlineStr">
         <is>
           <t>4pc Kiss-Cut Sticker Set Circle Ens Laptop Journal Bottle Zen Aesthetic Decal</t>
@@ -19264,8 +19712,16 @@
           <t>69fbaea961c4aefdea04aaaf</t>
         </is>
       </c>
-      <c r="F260" t="inlineStr"/>
-      <c r="G260" t="inlineStr"/>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>406909353931</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909353931</t>
+        </is>
+      </c>
       <c r="H260" t="inlineStr">
         <is>
           <t>Zen Aesthetic Praying Mantis on Rock 4pc 6x6 Kiss-Cut Sticker Laptop Journal</t>
@@ -19332,8 +19788,16 @@
           <t>69fbaeb9f60a24b6d1034575</t>
         </is>
       </c>
-      <c r="F261" t="inlineStr"/>
-      <c r="G261" t="inlineStr"/>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>406909354903</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909354903</t>
+        </is>
+      </c>
       <c r="H261" t="inlineStr">
         <is>
           <t>Mindful Zen Garden Stone Meis seki 4pc 6x6 Vinyl Sticker Laptop Journal Gift</t>
@@ -19400,8 +19864,16 @@
           <t>69fbaecbb8dd7e2bb0094b7c</t>
         </is>
       </c>
-      <c r="F262" t="inlineStr"/>
-      <c r="G262" t="inlineStr"/>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>406909355853</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909355853</t>
+        </is>
+      </c>
       <c r="H262" t="inlineStr">
         <is>
           <t>Mindful Zen Enso Circle with Crystals 4pc 6x6 Vinyl Sticker Laptop Journal Gift</t>
@@ -19468,8 +19940,16 @@
           <t>69fbaedb4c6544084c0f9620</t>
         </is>
       </c>
-      <c r="F263" t="inlineStr"/>
-      <c r="G263" t="inlineStr"/>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>406909359949</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909359949</t>
+        </is>
+      </c>
       <c r="H263" t="inlineStr">
         <is>
           <t>Koi Fish in Jade Pond Hisui no Koi Mindful Zen 4pc 6x6 Vinyl Sticker Yoga Luck</t>
@@ -19536,8 +20016,16 @@
           <t>69fbaeebce0d8cb5570fb7dc</t>
         </is>
       </c>
-      <c r="F264" t="inlineStr"/>
-      <c r="G264" t="inlineStr"/>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>406909364977</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909364977</t>
+        </is>
+      </c>
       <c r="H264" t="inlineStr">
         <is>
           <t>Minimal Zen Temple Lantern Zendera no T r 4pc 6x6 Sticker Sheet Serene Mindful</t>
@@ -19604,8 +20092,16 @@
           <t>69fbaefcc6dfbcc11107aa91</t>
         </is>
       </c>
-      <c r="F265" t="inlineStr"/>
-      <c r="G265" t="inlineStr"/>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>406909368739</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909368739</t>
+        </is>
+      </c>
       <c r="H265" t="inlineStr">
         <is>
           <t>Minimal Zen Kintsugi Gold Dragon 4pc 6x6 Sticker Sheet Serene Mindful Clean</t>
@@ -19672,8 +20168,16 @@
           <t>69fbaf12ff28e7d4030aba2d</t>
         </is>
       </c>
-      <c r="F266" t="inlineStr"/>
-      <c r="G266" t="inlineStr"/>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>406909373586</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909373586</t>
+        </is>
+      </c>
       <c r="H266" t="inlineStr">
         <is>
           <t>Bioluminescent Crystal Dragon Minimal Zen 4pc 6x6 Kiss-Cut Vinyl Desk Collector</t>
@@ -19740,8 +20244,16 @@
           <t>69fbc023f60a24b6d1034e5c</t>
         </is>
       </c>
-      <c r="F267" t="inlineStr"/>
-      <c r="G267" t="inlineStr"/>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>406909471020</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909471020</t>
+        </is>
+      </c>
       <c r="H267" t="inlineStr">
         <is>
           <t>Dark Academia Poster Theological Codex Sanctuary 12x18 Study Decor Wall Library</t>
@@ -19808,11 +20320,19 @@
           <t>69fbc0482b1da073620161ad</t>
         </is>
       </c>
-      <c r="F268" t="inlineStr"/>
-      <c r="G268" t="inlineStr"/>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>406909472775</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909472775</t>
+        </is>
+      </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t>Mechanical Encyclopedia Sphere Dark Academia Aesthetic 12x18 Poster Study Room</t>
+          <t>Reading Nook Smoky Jade Wall Art Mechanical 12x18 Matte Poster Apartment Decor</t>
         </is>
       </c>
       <c r="I268" t="inlineStr">
@@ -19842,7 +20362,7 @@
         <v>1</v>
       </c>
       <c r="S268" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T268" t="inlineStr">
         <is>
@@ -19944,7 +20464,7 @@
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>Printify_PublishExternalPending_Mockups8</t>
+          <t>Printify_Published_Mockups8</t>
         </is>
       </c>
       <c r="E270" t="inlineStr">
@@ -19952,8 +20472,16 @@
           <t>69fbccf9ce0d8cb5570fc6f0</t>
         </is>
       </c>
-      <c r="F270" t="inlineStr"/>
-      <c r="G270" t="inlineStr"/>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>406910056059</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406910056059</t>
+        </is>
+      </c>
       <c r="H270" t="inlineStr">
         <is>
           <t>Geological Archive Geode Dark Academia Poster 12x18 Mentor-Grade Decor Wall</t>
@@ -20012,7 +20540,7 @@
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>Printify_PublishExternalPending_Mockups8</t>
+          <t>Printify_Published_Mockups8</t>
         </is>
       </c>
       <c r="E271" t="inlineStr">
@@ -20020,8 +20548,16 @@
           <t>69fbcd1aee663532c8019ec7</t>
         </is>
       </c>
-      <c r="F271" t="inlineStr"/>
-      <c r="G271" t="inlineStr"/>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>406910057355</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406910057355</t>
+        </is>
+      </c>
       <c r="H271" t="inlineStr">
         <is>
           <t>Dark Academia Horological Manuscript Chamber Poster 12x18 Study Decor Wall Gift</t>
@@ -20080,7 +20616,7 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>Printify_PublishExternalPending_Mockups8</t>
+          <t>Printify_Published_Mockups8</t>
         </is>
       </c>
       <c r="E272" t="inlineStr">
@@ -20088,8 +20624,16 @@
           <t>69fbcd3eb8dd7e2bb0095af7</t>
         </is>
       </c>
-      <c r="F272" t="inlineStr"/>
-      <c r="G272" t="inlineStr"/>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>406910058626</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406910058626</t>
+        </is>
+      </c>
       <c r="H272" t="inlineStr">
         <is>
           <t>Dark Academia Meteorological Orrery 12x18 Poster Study Decor Atmospheric Texts</t>
@@ -20148,7 +20692,7 @@
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>Printify_PublishExternalPending_Mockups8</t>
+          <t>Printify_Published_Mockups8</t>
         </is>
       </c>
       <c r="E273" t="inlineStr">
@@ -20156,8 +20700,16 @@
           <t>69fbcd65cacc667dc70b7c2a</t>
         </is>
       </c>
-      <c r="F273" t="inlineStr"/>
-      <c r="G273" t="inlineStr"/>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>406910059060</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406910059060</t>
+        </is>
+      </c>
       <c r="H273" t="inlineStr">
         <is>
           <t>Dark Academia Astrological Globe Poster 12x18 Study Room Decor Starlight Jade</t>
@@ -20216,7 +20768,7 @@
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>Printify_PublishExternalPending_Mockups8</t>
+          <t>Printify_Published_Mockups8</t>
         </is>
       </c>
       <c r="E274" t="inlineStr">
@@ -20224,8 +20776,16 @@
           <t>69fbcd8a3014a1ea840da971</t>
         </is>
       </c>
-      <c r="F274" t="inlineStr"/>
-      <c r="G274" t="inlineStr"/>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>406910060084</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406910060084</t>
+        </is>
+      </c>
       <c r="H274" t="inlineStr">
         <is>
           <t>Dark Academia Armillary Sphere Poster 12x18 Vintage Study Decor Zodiac Symbols</t>

</xml_diff>

<commit_message>
Refine live gallery integrity gate
</commit_message>
<xml_diff>
--- a/Database/Unified_Listing_Registry.xlsx
+++ b/Database/Unified_Listing_Registry.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Unified Registry" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Unified Registry'!$A$1:$T$283</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Unified Registry'!$A$1:$T$300</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T283"/>
+  <dimension ref="A1:T300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -740,7 +740,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -4600,7 +4600,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -4666,7 +4666,7 @@
       </c>
       <c r="T59" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -4688,7 +4688,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -4754,7 +4754,7 @@
       </c>
       <c r="T60" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -4842,7 +4842,7 @@
       </c>
       <c r="T61" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -4864,7 +4864,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -4930,7 +4930,7 @@
       </c>
       <c r="T62" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -4952,7 +4952,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -5018,7 +5018,7 @@
       </c>
       <c r="T63" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -5040,7 +5040,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -5106,7 +5106,7 @@
       </c>
       <c r="T64" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -5128,7 +5128,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -5194,7 +5194,7 @@
       </c>
       <c r="T65" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -5216,7 +5216,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -5282,7 +5282,7 @@
       </c>
       <c r="T66" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -5304,7 +5304,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -5516,7 +5516,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -5592,7 +5592,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -5668,7 +5668,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -10800,7 +10800,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
@@ -10866,7 +10866,7 @@
       </c>
       <c r="T151" t="inlineStr">
         <is>
-          <t>Published_Has_View_Monitor</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -10976,7 +10976,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
@@ -11050,7 +11050,7 @@
       </c>
       <c r="T153" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Etsy_Draft_Prepared</t>
         </is>
       </c>
     </row>
@@ -11072,7 +11072,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
@@ -11146,7 +11146,7 @@
       </c>
       <c r="T154" t="inlineStr">
         <is>
-          <t>Published_Has_View_Monitor</t>
+          <t>Etsy_Draft_Prepared</t>
         </is>
       </c>
     </row>
@@ -11168,7 +11168,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
@@ -11234,7 +11234,7 @@
       </c>
       <c r="T155" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -11256,7 +11256,7 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
@@ -11330,7 +11330,7 @@
       </c>
       <c r="T156" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Etsy_Draft_Prepared</t>
         </is>
       </c>
     </row>
@@ -11352,7 +11352,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
@@ -11426,7 +11426,7 @@
       </c>
       <c r="T157" t="inlineStr">
         <is>
-          <t>Published_Has_View_Monitor</t>
+          <t>Etsy_Draft_Prepared</t>
         </is>
       </c>
     </row>
@@ -11448,7 +11448,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
@@ -11514,7 +11514,7 @@
       </c>
       <c r="T158" t="inlineStr">
         <is>
-          <t>Published_Has_View_Monitor</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -11536,7 +11536,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
@@ -11610,7 +11610,7 @@
       </c>
       <c r="T159" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Etsy_Draft_Prepared</t>
         </is>
       </c>
     </row>
@@ -11632,7 +11632,7 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
@@ -11698,7 +11698,7 @@
       </c>
       <c r="T160" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -11720,7 +11720,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
@@ -11786,7 +11786,7 @@
       </c>
       <c r="T161" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -11808,7 +11808,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
@@ -11882,7 +11882,7 @@
       </c>
       <c r="T162" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Etsy_Draft_Prepared</t>
         </is>
       </c>
     </row>
@@ -11904,7 +11904,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
@@ -11970,7 +11970,7 @@
       </c>
       <c r="T163" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -11992,7 +11992,7 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
@@ -12058,7 +12058,7 @@
       </c>
       <c r="T164" t="inlineStr">
         <is>
-          <t>Published_Has_View_Monitor</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -12080,7 +12080,7 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
@@ -12154,7 +12154,7 @@
       </c>
       <c r="T165" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Etsy_Draft_Prepared</t>
         </is>
       </c>
     </row>
@@ -12176,7 +12176,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
@@ -12242,7 +12242,7 @@
       </c>
       <c r="T166" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -12264,7 +12264,7 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
@@ -12330,7 +12330,7 @@
       </c>
       <c r="T167" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -12352,7 +12352,7 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
@@ -12418,7 +12418,7 @@
       </c>
       <c r="T168" t="inlineStr">
         <is>
-          <t>Published_Has_View_Monitor</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -12440,7 +12440,7 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
@@ -12506,7 +12506,7 @@
       </c>
       <c r="T169" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -12528,7 +12528,7 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E170" t="inlineStr">
@@ -12594,7 +12594,7 @@
       </c>
       <c r="T170" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -12616,7 +12616,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
@@ -12690,7 +12690,7 @@
       </c>
       <c r="T171" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Etsy_Draft_Prepared</t>
         </is>
       </c>
     </row>
@@ -12776,7 +12776,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
@@ -12850,7 +12850,7 @@
       </c>
       <c r="T173" t="inlineStr">
         <is>
-          <t>Published_Has_View_Monitor</t>
+          <t>Etsy_Draft_Prepared</t>
         </is>
       </c>
     </row>
@@ -12872,7 +12872,7 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
@@ -12946,7 +12946,7 @@
       </c>
       <c r="T174" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Etsy_Draft_Prepared</t>
         </is>
       </c>
     </row>
@@ -12968,7 +12968,7 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
@@ -13034,7 +13034,7 @@
       </c>
       <c r="T175" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -13056,7 +13056,7 @@
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
@@ -13130,7 +13130,7 @@
       </c>
       <c r="T176" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Etsy_Draft_Prepared</t>
         </is>
       </c>
     </row>
@@ -13152,7 +13152,7 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
@@ -13172,12 +13172,12 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>Quiet Luxury Apartment Art Phoenix Rebirth Vessel for Meditation 12x18 Matte</t>
+          <t>Quiet Luxury Jade Wall Art Reading Nook 12x18 Matte Poster Apartment Decor Gift</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>$34.99</t>
+          <t>$29.99</t>
         </is>
       </c>
       <c r="J177" t="inlineStr">
@@ -13218,7 +13218,7 @@
       </c>
       <c r="T177" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -13796,12 +13796,12 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>Quiet Luxury Shelf Decor Necromancer Soul Reliquary Artifact 5x7 Acrylic Photo</t>
+          <t>Collector Shelf Smoky Jade Quiet Luxury 5x7 Acrylic Block Shelf Decor Gift Wall</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>$89.99</t>
+          <t>$84.99</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
@@ -13892,9 +13892,21 @@
           <t>$89.99</t>
         </is>
       </c>
-      <c r="J185" t="inlineStr"/>
-      <c r="K185" t="inlineStr"/>
-      <c r="L185" t="inlineStr"/>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M185" t="b">
         <v>0</v>
       </c>
@@ -13918,7 +13930,7 @@
       </c>
       <c r="T185" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -13968,9 +13980,21 @@
           <t>$89.99</t>
         </is>
       </c>
-      <c r="J186" t="inlineStr"/>
-      <c r="K186" t="inlineStr"/>
-      <c r="L186" t="inlineStr"/>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K186" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M186" t="b">
         <v>0</v>
       </c>
@@ -13994,7 +14018,7 @@
       </c>
       <c r="T186" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -14036,17 +14060,29 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>Gothic Grimdark Revenant Lantern 5x7 Acrylic Art Premium Decor Sapphire Glass</t>
+          <t>Quiet Luxury Jade Relic Revenant 5x7 Acrylic Block Shelf Decor Gift Study Wall</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>$89.99</t>
-        </is>
-      </c>
-      <c r="J187" t="inlineStr"/>
-      <c r="K187" t="inlineStr"/>
-      <c r="L187" t="inlineStr"/>
+          <t>$84.99</t>
+        </is>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M187" t="b">
         <v>0</v>
       </c>
@@ -14066,11 +14102,11 @@
         <v>1</v>
       </c>
       <c r="S187" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T187" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -14120,9 +14156,21 @@
           <t>$89.99</t>
         </is>
       </c>
-      <c r="J188" t="inlineStr"/>
-      <c r="K188" t="inlineStr"/>
-      <c r="L188" t="inlineStr"/>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M188" t="b">
         <v>0</v>
       </c>
@@ -14146,7 +14194,7 @@
       </c>
       <c r="T188" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -14188,17 +14236,29 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>Gothic Wraith Warden Cursed Beacon 5x7 Acrylic Block Dark Fantasy Decor Shelf</t>
+          <t>Collector Shelf Smoky Jade Wraith Warden 5x7 Acrylic Block Shelf Decor Gift</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>$89.99</t>
-        </is>
-      </c>
-      <c r="J189" t="inlineStr"/>
-      <c r="K189" t="inlineStr"/>
-      <c r="L189" t="inlineStr"/>
+          <t>$84.99</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M189" t="b">
         <v>0</v>
       </c>
@@ -14218,11 +14278,11 @@
         <v>1</v>
       </c>
       <c r="S189" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T189" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -14448,12 +14508,12 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>Reading Nook Wall Decor Mystic Threshold Infinite Knowledge 12x18 Matte Poster</t>
+          <t>Dark Academia Reading Nook Art Mystic Threshold Infinite 12x18 Matte Poster</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>$34.99</t>
+          <t>$29.99</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
@@ -14920,9 +14980,21 @@
           <t>$34.99</t>
         </is>
       </c>
-      <c r="J197" t="inlineStr"/>
-      <c r="K197" t="inlineStr"/>
-      <c r="L197" t="inlineStr"/>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M197" t="b">
         <v>0</v>
       </c>
@@ -14946,7 +15018,7 @@
       </c>
       <c r="T197" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -14996,9 +15068,21 @@
           <t>$89.99</t>
         </is>
       </c>
-      <c r="J198" t="inlineStr"/>
-      <c r="K198" t="inlineStr"/>
-      <c r="L198" t="inlineStr"/>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M198" t="b">
         <v>0</v>
       </c>
@@ -15022,7 +15106,7 @@
       </c>
       <c r="T198" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -15368,12 +15452,12 @@
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>Gothic Grimdark Shadowpriest Ritual Vessel 5x7 Acrylic Decor Indigo Flame Shelf</t>
+          <t>Quiet Luxury Jade Relic Shadowpriest 5x7 Acrylic Block Shelf Decor Gift Study</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
         <is>
-          <t>$89.99</t>
+          <t>$84.99</t>
         </is>
       </c>
       <c r="J203" t="inlineStr"/>
@@ -15398,7 +15482,7 @@
         <v>1</v>
       </c>
       <c r="S203" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T203" t="inlineStr">
         <is>
@@ -16280,12 +16364,12 @@
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>Spectral Temple Soul Lantern Grimdark Mentor-Grade 5x7 Acrylic Art Collectible</t>
+          <t>Quiet Luxury Jade Relic Spectral 5x7 Acrylic Block Shelf Decor Gift Study Wall</t>
         </is>
       </c>
       <c r="I215" t="inlineStr">
         <is>
-          <t>$89.99</t>
+          <t>$84.99</t>
         </is>
       </c>
       <c r="J215" t="inlineStr"/>
@@ -16310,7 +16394,7 @@
         <v>1</v>
       </c>
       <c r="S215" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T215" t="inlineStr">
         <is>
@@ -16356,12 +16440,12 @@
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>Midnight Sanctuary Soul Lantern Grimdark 5x7 Acrylic Collectible Display Shelf</t>
+          <t>Collector Shelf Smoky Jade Midnight Sanctuary 5x7 Acrylic Block Shelf Decor</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
         <is>
-          <t>$89.99</t>
+          <t>$84.99</t>
         </is>
       </c>
       <c r="J216" t="inlineStr"/>
@@ -16386,7 +16470,7 @@
         <v>1</v>
       </c>
       <c r="S216" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T216" t="inlineStr">
         <is>
@@ -16660,12 +16744,12 @@
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>Twilight Portal Soul Lantern Grimdark 5x7 Acrylic Art Gothic Decor Purple Flame</t>
+          <t>Quiet Luxury Jade Relic Twilight 5x7 Acrylic Block Shelf Decor Gift Study Wall</t>
         </is>
       </c>
       <c r="I220" t="inlineStr">
         <is>
-          <t>$89.99</t>
+          <t>$84.99</t>
         </is>
       </c>
       <c r="J220" t="inlineStr"/>
@@ -16690,7 +16774,7 @@
         <v>1</v>
       </c>
       <c r="S220" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T220" t="inlineStr">
         <is>
@@ -16964,12 +17048,12 @@
       </c>
       <c r="H224" t="inlineStr">
         <is>
-          <t>Smoky Jade Gothic Object Sapphire Temple Soul Lantern Artifact 5x7 Acrylic Gift</t>
+          <t>Quiet Luxury Jade Relic Smoky 5x7 Acrylic Block Shelf Decor Gift Study Wall</t>
         </is>
       </c>
       <c r="I224" t="inlineStr">
         <is>
-          <t>$89.99</t>
+          <t>$84.99</t>
         </is>
       </c>
       <c r="J224" t="inlineStr"/>
@@ -17124,9 +17208,21 @@
           <t>$34.99</t>
         </is>
       </c>
-      <c r="J226" t="inlineStr"/>
-      <c r="K226" t="inlineStr"/>
-      <c r="L226" t="inlineStr"/>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K226" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L226" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M226" t="b">
         <v>0</v>
       </c>
@@ -17150,7 +17246,7 @@
       </c>
       <c r="T226" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -17200,9 +17296,21 @@
           <t>$34.99</t>
         </is>
       </c>
-      <c r="J227" t="inlineStr"/>
-      <c r="K227" t="inlineStr"/>
-      <c r="L227" t="inlineStr"/>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K227" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L227" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M227" t="b">
         <v>0</v>
       </c>
@@ -17226,7 +17334,7 @@
       </c>
       <c r="T227" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -17276,9 +17384,21 @@
           <t>$34.99</t>
         </is>
       </c>
-      <c r="J228" t="inlineStr"/>
-      <c r="K228" t="inlineStr"/>
-      <c r="L228" t="inlineStr"/>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K228" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L228" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M228" t="b">
         <v>0</v>
       </c>
@@ -17302,7 +17422,7 @@
       </c>
       <c r="T228" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -17352,9 +17472,21 @@
           <t>$34.99</t>
         </is>
       </c>
-      <c r="J229" t="inlineStr"/>
-      <c r="K229" t="inlineStr"/>
-      <c r="L229" t="inlineStr"/>
+      <c r="J229" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K229" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L229" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M229" t="b">
         <v>1</v>
       </c>
@@ -17386,7 +17518,7 @@
       </c>
       <c r="T229" t="inlineStr">
         <is>
-          <t>Etsy_Draft_Prepared</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -17436,9 +17568,21 @@
           <t>$34.99</t>
         </is>
       </c>
-      <c r="J230" t="inlineStr"/>
-      <c r="K230" t="inlineStr"/>
-      <c r="L230" t="inlineStr"/>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K230" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="L230" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
       <c r="M230" t="b">
         <v>0</v>
       </c>
@@ -17462,7 +17606,7 @@
       </c>
       <c r="T230" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
     </row>
@@ -21510,8 +21654,1300 @@
         </is>
       </c>
     </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0055-FIX1</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Printify_Published_Mockups3</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>69fcad74346e75ac9f07d550</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>406910984204</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406910984204</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>Quiet Desk Sticker Pack Azure Dragon Warrior 4pc 6x6 Kiss-Cut Vinyl Laptop Gift</t>
+        </is>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>$11.99</t>
+        </is>
+      </c>
+      <c r="J284" t="inlineStr"/>
+      <c r="K284" t="inlineStr"/>
+      <c r="L284" t="inlineStr"/>
+      <c r="M284" t="b">
+        <v>0</v>
+      </c>
+      <c r="N284" t="inlineStr"/>
+      <c r="O284" t="inlineStr"/>
+      <c r="P284" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0055_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="Q284" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0055_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="R284" t="b">
+        <v>1</v>
+      </c>
+      <c r="S284" t="b">
+        <v>0</v>
+      </c>
+      <c r="T284" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0056-FIX1</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Printify_Published_Mockups3</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>69fcb688d0e6f406f20a3d2a</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>406911030956</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911030956</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>Reading Nook Vinyl Set Dragon Cherry Blossom 4pc 6x6 Kiss-Cut Vinyl Laptop Gift</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>$11.99</t>
+        </is>
+      </c>
+      <c r="J285" t="inlineStr"/>
+      <c r="K285" t="inlineStr"/>
+      <c r="L285" t="inlineStr"/>
+      <c r="M285" t="b">
+        <v>0</v>
+      </c>
+      <c r="N285" t="inlineStr"/>
+      <c r="O285" t="inlineStr"/>
+      <c r="P285" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0056_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="Q285" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0056_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="R285" t="b">
+        <v>1</v>
+      </c>
+      <c r="S285" t="b">
+        <v>0</v>
+      </c>
+      <c r="T285" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0057-FIX1</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Printify_Published</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>69fcb8762007fddea00e4ebe</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>406911046712</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911046712</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>Wabi Sabi Journal Decals Moonlit Dragon 4pc 6x6 Kiss-Cut Vinyl Laptop Journal</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>$11.99</t>
+        </is>
+      </c>
+      <c r="J286" t="inlineStr"/>
+      <c r="K286" t="inlineStr"/>
+      <c r="L286" t="inlineStr"/>
+      <c r="M286" t="b">
+        <v>0</v>
+      </c>
+      <c r="N286" t="inlineStr"/>
+      <c r="O286" t="inlineStr"/>
+      <c r="P286" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0057_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="Q286" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0057_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="R286" t="b">
+        <v>1</v>
+      </c>
+      <c r="S286" t="b">
+        <v>0</v>
+      </c>
+      <c r="T286" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0058-FIX1</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Printify_Published</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>69fcbabcbb3409c48f0e342c</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>406911102240</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911102240</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>Smoky Jade Sticker Set Dragon Calligraphy Serene Clean 4pc 6x6 Kiss-Cut Vinyl</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>$11.99</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr"/>
+      <c r="K287" t="inlineStr"/>
+      <c r="L287" t="inlineStr"/>
+      <c r="M287" t="b">
+        <v>0</v>
+      </c>
+      <c r="N287" t="inlineStr"/>
+      <c r="O287" t="inlineStr"/>
+      <c r="P287" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0058_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="Q287" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0058_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="R287" t="b">
+        <v>1</v>
+      </c>
+      <c r="S287" t="b">
+        <v>0</v>
+      </c>
+      <c r="T287" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0060-FIX1</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Printify_Published</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>69fcc02e6a069c45c0013c52</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>406911120974</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911120974</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>Reading Nook Vinyl Set Translucent Jade Dragon Serene Clean 4pc 6x6 Kiss-Cut</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>$11.99</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr"/>
+      <c r="K288" t="inlineStr"/>
+      <c r="L288" t="inlineStr"/>
+      <c r="M288" t="b">
+        <v>0</v>
+      </c>
+      <c r="N288" t="inlineStr"/>
+      <c r="O288" t="inlineStr"/>
+      <c r="P288" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0060_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="Q288" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0060_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="R288" t="b">
+        <v>1</v>
+      </c>
+      <c r="S288" t="b">
+        <v>0</v>
+      </c>
+      <c r="T288" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0061-FIX1</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Printify_Published_Mockups3</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>69fcf2ccf2b2884ff107c609</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>406911452547</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911452547</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>Wabi Sabi Journal Decals Kintsugi Gold Dragon Serene Calm 4pc 6x6 Kiss-Cut Gift</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>$11.99</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr"/>
+      <c r="K289" t="inlineStr"/>
+      <c r="L289" t="inlineStr"/>
+      <c r="M289" t="b">
+        <v>0</v>
+      </c>
+      <c r="N289" t="inlineStr"/>
+      <c r="O289" t="inlineStr"/>
+      <c r="P289" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0061_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="Q289" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0061_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="R289" t="b">
+        <v>1</v>
+      </c>
+      <c r="S289" t="b">
+        <v>0</v>
+      </c>
+      <c r="T289" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0062-FIX1</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Printify_Published_Mockups3</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>69fcfa3363b7f727e7012b1a</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>406911488570</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911488570</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>Smoky Jade Sticker Set Bioluminescent Dragon 4pc 6x6 Kiss-Cut Vinyl Laptop Gift</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>$11.99</t>
+        </is>
+      </c>
+      <c r="J290" t="inlineStr"/>
+      <c r="K290" t="inlineStr"/>
+      <c r="L290" t="inlineStr"/>
+      <c r="M290" t="b">
+        <v>0</v>
+      </c>
+      <c r="N290" t="inlineStr"/>
+      <c r="O290" t="inlineStr"/>
+      <c r="P290" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0062_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="Q290" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0062_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="R290" t="b">
+        <v>1</v>
+      </c>
+      <c r="S290" t="b">
+        <v>0</v>
+      </c>
+      <c r="T290" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0063-FIX1</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Printify_Published_Mockups3</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>69fcfb2d111bf518b6078098</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>406911494155</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911494155</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>Crystalline Dragon Core 4pc 6x6 Kiss-Cut Sticker Zen Aesthetic Laptop Journal</t>
+        </is>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>$11.99</t>
+        </is>
+      </c>
+      <c r="J291" t="inlineStr"/>
+      <c r="K291" t="inlineStr"/>
+      <c r="L291" t="inlineStr"/>
+      <c r="M291" t="b">
+        <v>0</v>
+      </c>
+      <c r="N291" t="inlineStr"/>
+      <c r="O291" t="inlineStr"/>
+      <c r="P291" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0063_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="Q291" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0063_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="R291" t="b">
+        <v>1</v>
+      </c>
+      <c r="S291" t="b">
+        <v>1</v>
+      </c>
+      <c r="T291" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0066-FIX1</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Printify_Published_Mockups3</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>69fcfd2914568b768c07abd9</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>406911509730</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911509730</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>Golden Vein Circuitry Dragon 4pc 6x6 Kiss-Cut Sticker Zen Aesthetic Laptop Gift</t>
+        </is>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>$11.99</t>
+        </is>
+      </c>
+      <c r="J292" t="inlineStr"/>
+      <c r="K292" t="inlineStr"/>
+      <c r="L292" t="inlineStr"/>
+      <c r="M292" t="b">
+        <v>0</v>
+      </c>
+      <c r="N292" t="inlineStr"/>
+      <c r="O292" t="inlineStr"/>
+      <c r="P292" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0066_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="Q292" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0066_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="R292" t="b">
+        <v>1</v>
+      </c>
+      <c r="S292" t="b">
+        <v>1</v>
+      </c>
+      <c r="T292" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0069-FIX1</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Printify_Published_Mockups3</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>69fcff15cd220b844e0f655c</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>406911531255</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911531255</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>Minimal Zen Dragon Guardian 4pc 6x6 Sticker Sheet Serene Mindful Clean Decor</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>$11.99</t>
+        </is>
+      </c>
+      <c r="J293" t="inlineStr"/>
+      <c r="K293" t="inlineStr"/>
+      <c r="L293" t="inlineStr"/>
+      <c r="M293" t="b">
+        <v>0</v>
+      </c>
+      <c r="N293" t="inlineStr"/>
+      <c r="O293" t="inlineStr"/>
+      <c r="P293" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0069_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="Q293" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0069_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="R293" t="b">
+        <v>1</v>
+      </c>
+      <c r="S293" t="b">
+        <v>1</v>
+      </c>
+      <c r="T293" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0070-FIX1</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Printify_Published_Mockups3</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>69fd002f096d6b4f0000a934</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>406911541926</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911541926</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>Minimal Zen Jade Phoenix Ascension 4pc 6x6 Sticker Sheet Serene Mindful Clean</t>
+        </is>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>$11.99</t>
+        </is>
+      </c>
+      <c r="J294" t="inlineStr"/>
+      <c r="K294" t="inlineStr"/>
+      <c r="L294" t="inlineStr"/>
+      <c r="M294" t="b">
+        <v>0</v>
+      </c>
+      <c r="N294" t="inlineStr"/>
+      <c r="O294" t="inlineStr"/>
+      <c r="P294" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0070_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="Q294" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0070_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="R294" t="b">
+        <v>1</v>
+      </c>
+      <c r="S294" t="b">
+        <v>1</v>
+      </c>
+      <c r="T294" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0071-FIX1</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Printify_Published_Mockups3</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>69fd00ca9f7703138202688c</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>406911551031</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911551031</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>Zen Aesthetic Lotus Lantern Vessel 4pc 6x6 Kiss-Cut Sticker Laptop Journal Gift</t>
+        </is>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>$11.99</t>
+        </is>
+      </c>
+      <c r="J295" t="inlineStr"/>
+      <c r="K295" t="inlineStr"/>
+      <c r="L295" t="inlineStr"/>
+      <c r="M295" t="b">
+        <v>0</v>
+      </c>
+      <c r="N295" t="inlineStr"/>
+      <c r="O295" t="inlineStr"/>
+      <c r="P295" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0071_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="Q295" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0071_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="R295" t="b">
+        <v>1</v>
+      </c>
+      <c r="S295" t="b">
+        <v>1</v>
+      </c>
+      <c r="T295" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0081-FIX1</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Acrylic</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>Grimdark</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Printify_Published_Mockups4</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>69fd02f3d70cf705c50f4d27</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>406911568594</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911568594</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>Smoky Jade Desk Object Plague Doctor Raven Skull Alchemy 5x7 Acrylic Photo Gift</t>
+        </is>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>$89.99</t>
+        </is>
+      </c>
+      <c r="J296" t="inlineStr"/>
+      <c r="K296" t="inlineStr"/>
+      <c r="L296" t="inlineStr"/>
+      <c r="M296" t="b">
+        <v>0</v>
+      </c>
+      <c r="N296" t="inlineStr"/>
+      <c r="O296" t="inlineStr"/>
+      <c r="P296" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0081_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="Q296" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0081_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="R296" t="b">
+        <v>1</v>
+      </c>
+      <c r="S296" t="b">
+        <v>0</v>
+      </c>
+      <c r="T296" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>Acrylic-Zen-0001-FIX1</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Acrylic</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Printify_Published_Mockups4</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>69fd040f6873b551670941bd</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>406911574121</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911574121</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>Smoky Jade Desk Object Mechanical Crane Calm Origami Sculpture 5x7 Acrylic Gift</t>
+        </is>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>$89.99</t>
+        </is>
+      </c>
+      <c r="J297" t="inlineStr"/>
+      <c r="K297" t="inlineStr"/>
+      <c r="L297" t="inlineStr"/>
+      <c r="M297" t="b">
+        <v>0</v>
+      </c>
+      <c r="N297" t="inlineStr"/>
+      <c r="O297" t="inlineStr"/>
+      <c r="P297" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Zen-0001_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="Q297" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Zen-0001_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="R297" t="b">
+        <v>1</v>
+      </c>
+      <c r="S297" t="b">
+        <v>0</v>
+      </c>
+      <c r="T297" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0001-FIX1</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Poster</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>Academia</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Printify_Published</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>69fd05fcd70cf705c50f4ef9</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>406911589289</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911589289</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>Celestial Gateway Dark Academia Poster 12x18 Study Decor Moonstone Architecture</t>
+        </is>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>$34.99</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr"/>
+      <c r="K298" t="inlineStr"/>
+      <c r="L298" t="inlineStr"/>
+      <c r="M298" t="b">
+        <v>0</v>
+      </c>
+      <c r="N298" t="inlineStr"/>
+      <c r="O298" t="inlineStr"/>
+      <c r="P298" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0001_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="Q298" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0001_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="R298" t="b">
+        <v>1</v>
+      </c>
+      <c r="S298" t="b">
+        <v>1</v>
+      </c>
+      <c r="T298" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0003-FIX1</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Poster</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>Academia</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>Printify_Published</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>69fd095c9f77031382026de2</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>406911598735</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911598735</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>Reading Nook Wall Decor Serpentine Portal of Alchemical Texts 12x18 Matte Gift</t>
+        </is>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>$34.99</t>
+        </is>
+      </c>
+      <c r="J299" t="inlineStr"/>
+      <c r="K299" t="inlineStr"/>
+      <c r="L299" t="inlineStr"/>
+      <c r="M299" t="b">
+        <v>0</v>
+      </c>
+      <c r="N299" t="inlineStr"/>
+      <c r="O299" t="inlineStr"/>
+      <c r="P299" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0003_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="Q299" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0003_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="R299" t="b">
+        <v>1</v>
+      </c>
+      <c r="S299" t="b">
+        <v>0</v>
+      </c>
+      <c r="T299" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>Acrylic-Academia-0003-GALLERYFIX1</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>Acrylic</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>Academia</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>Printify_Published_Mockups4</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>69fd36d2a4235c1793034b29</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>406911883288</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911883288</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>Quiet Luxury Shelf Decor Celestial Orrery Tree Bonsai 5x7 Acrylic Photo Block</t>
+        </is>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>$89.99</t>
+        </is>
+      </c>
+      <c r="J300" t="inlineStr"/>
+      <c r="K300" t="inlineStr"/>
+      <c r="L300" t="inlineStr"/>
+      <c r="M300" t="b">
+        <v>0</v>
+      </c>
+      <c r="N300" t="inlineStr"/>
+      <c r="O300" t="inlineStr"/>
+      <c r="P300" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Academia-0003_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="Q300" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Academia-0003_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="R300" t="b">
+        <v>1</v>
+      </c>
+      <c r="S300" t="b">
+        <v>0</v>
+      </c>
+      <c r="T300" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T283"/>
+  <autoFilter ref="A1:T300"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refresh monthly factory state
</commit_message>
<xml_diff>
--- a/Database/Unified_Listing_Registry.xlsx
+++ b/Database/Unified_Listing_Registry.xlsx
@@ -2180,7 +2180,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -5744,7 +5744,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -5820,7 +5820,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -5896,7 +5896,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -5972,7 +5972,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups4</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -6448,14 +6448,10 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups5</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>69f2683ecaeb1241880b7fcb</t>
-        </is>
-      </c>
+          <t>Ready_for_Printify</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
@@ -6494,7 +6490,7 @@
       </c>
       <c r="T83" t="inlineStr">
         <is>
-          <t>Stable_Draft_Publish_When_Scheduled</t>
+          <t>Ready_For_Printify_When_Network_OK</t>
         </is>
       </c>
     </row>
@@ -6516,7 +6512,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -6562,7 +6558,7 @@
       </c>
       <c r="T84" t="inlineStr">
         <is>
-          <t>Stable_Draft_Publish_When_Scheduled</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -6648,7 +6644,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -6694,7 +6690,7 @@
       </c>
       <c r="T86" t="inlineStr">
         <is>
-          <t>Stable_Draft_Publish_When_Scheduled</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -6716,7 +6712,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -6762,7 +6758,7 @@
       </c>
       <c r="T87" t="inlineStr">
         <is>
-          <t>Stable_Draft_Publish_When_Scheduled</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -6784,7 +6780,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -6830,7 +6826,7 @@
       </c>
       <c r="T88" t="inlineStr">
         <is>
-          <t>Stable_Draft_Publish_When_Scheduled</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -6852,7 +6848,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -6898,7 +6894,7 @@
       </c>
       <c r="T89" t="inlineStr">
         <is>
-          <t>Stable_Draft_Publish_When_Scheduled</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -6984,7 +6980,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -7030,7 +7026,7 @@
       </c>
       <c r="T91" t="inlineStr">
         <is>
-          <t>Stable_Draft_Publish_When_Scheduled</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -7052,7 +7048,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -7098,7 +7094,7 @@
       </c>
       <c r="T92" t="inlineStr">
         <is>
-          <t>Stable_Draft_Publish_When_Scheduled</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -7120,7 +7116,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -7166,7 +7162,7 @@
       </c>
       <c r="T93" t="inlineStr">
         <is>
-          <t>Stable_Draft_Publish_When_Scheduled</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -7188,7 +7184,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -7234,7 +7230,7 @@
       </c>
       <c r="T94" t="inlineStr">
         <is>
-          <t>Stable_Draft_Publish_When_Scheduled</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -10928,7 +10924,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
@@ -10994,7 +10990,7 @@
       </c>
       <c r="T152" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
     </row>
@@ -11964,7 +11960,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>Deep Work Desk Visual Pagoda Fragment Relic Print Floating 5x7 Acrylic Photo</t>
+          <t>Meditation Room Jade Relic Deep Work Visual Pagoda 5x7 Acrylic Block Shelf Gift</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -12500,7 +12496,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>Gallery Desk Art Incense Vessel Constellation for Meditation 5x7 Acrylic Photo</t>
+          <t>Meditation Room Jade Relic Incense Vessel Constellation 5x7 Acrylic Block Decor</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -13660,7 +13656,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>Deep Work Desk Visual Lantern Soul Cage Crimson Flame 5x7 Acrylic Photo Block</t>
+          <t>Dark Study Smoky Jade Deep Work Visual Lantern 5x7 Acrylic Block Shelf Decor</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -14188,7 +14184,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>Gothic Grimdark Lich Phylactery Lantern 5x7 Acrylic Print Dark Fantasy Home</t>
+          <t>Quiet Luxury Jade Relic Lich Phylactery Lantern Fantasy 5x7 Acrylic Block Decor</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -14230,7 +14226,7 @@
         <v>1</v>
       </c>
       <c r="S188" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T188" t="inlineStr">
         <is>
@@ -15568,7 +15564,7 @@
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>Grimdark Aesthetic Dreadlord Beacon Lantern 5x7 Acrylic Block Dark Decor Shelf</t>
+          <t>Collector Shelf Smoky Jade Dreadlord Beacon Lantern 5x7 Acrylic Block Shelf</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
@@ -15598,7 +15594,7 @@
         <v>1</v>
       </c>
       <c r="S204" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T204" t="inlineStr">
         <is>
@@ -15872,7 +15868,7 @@
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>Violet Torment Lantern 5x7 Acrylic Grimdark Gothic Decor for Dark Fantasy Study</t>
+          <t>Dark Study Smoky Jade Violet Torment Lantern Fantasy 5x7 Acrylic Block Shelf</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
@@ -15902,7 +15898,7 @@
         <v>1</v>
       </c>
       <c r="S208" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T208" t="inlineStr">
         <is>
@@ -16480,12 +16476,12 @@
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>Collector Shelf Smoky Jade Midnight Sanctuary 5x7 Acrylic Block Shelf Decor</t>
+          <t>Quiet Luxury Jade Relic Collector Smoky Midnight Sanctuary 5x7 Acrylic Block</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
         <is>
-          <t>$84.99</t>
+          <t>$89.99</t>
         </is>
       </c>
       <c r="J216" t="inlineStr"/>
@@ -16556,7 +16552,7 @@
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>Grimdark Amber Monastery Soul Lantern 5x7 Acrylic Art Gothic Decor Golden Flame</t>
+          <t>Collector Shelf Smoky Jade Amber Monastery Soul Lantern 5x7 Acrylic Block Decor</t>
         </is>
       </c>
       <c r="I217" t="inlineStr">
@@ -16586,7 +16582,7 @@
         <v>1</v>
       </c>
       <c r="S217" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T217" t="inlineStr">
         <is>
@@ -16860,7 +16856,7 @@
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>Gothic Frost Cathedral Soul Lantern 5x7 Acrylic Display Grimdark Artifact Shelf</t>
+          <t>Quiet Luxury Jade Relic Frost Cathedral Soul Lantern 5x7 Acrylic Block Shelf</t>
         </is>
       </c>
       <c r="I221" t="inlineStr">
@@ -16890,7 +16886,7 @@
         <v>1</v>
       </c>
       <c r="S221" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T221" t="inlineStr">
         <is>
@@ -17688,7 +17684,7 @@
       </c>
       <c r="H231" t="inlineStr">
         <is>
-          <t>Hermetic Knowledge Lantern Dark Academia Poster 12x18 Library Decor Wall Study</t>
+          <t>Dark Academia Reading Nook Art Hermetic Knowledge Lantern Library 12x18 Matte</t>
         </is>
       </c>
       <c r="I231" t="inlineStr">
@@ -17718,7 +17714,7 @@
         <v>1</v>
       </c>
       <c r="S231" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T231" t="inlineStr">
         <is>

</xml_diff>